<commit_message>
Update model outputs 2026-10-18 22:23:55
</commit_message>
<xml_diff>
--- a/files/A-Leagues_upcoming_projections.xlsx
+++ b/files/A-Leagues_upcoming_projections.xlsx
@@ -357,7 +357,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BT15"/>
+  <dimension ref="A1:BT9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -882,7 +882,7 @@
       </c>
       <c r="AQ2" t="inlineStr">
         <is>
-          <t>2026-10-18 11:46:55 AEDT</t>
+          <t>2026-10-18 13:43:17 AEDT</t>
         </is>
       </c>
       <c r="AR2" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="AQ3" t="inlineStr">
         <is>
-          <t>2026-10-18 11:46:55 AEDT</t>
+          <t>2026-10-18 13:43:17 AEDT</t>
         </is>
       </c>
       <c r="AR3" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="AQ4" t="inlineStr">
         <is>
-          <t>2026-10-18 11:46:55 AEDT</t>
+          <t>2026-10-18 13:43:17 AEDT</t>
         </is>
       </c>
       <c r="AR4" t="inlineStr">
@@ -1674,7 +1674,7 @@
       </c>
       <c r="AQ5" t="inlineStr">
         <is>
-          <t>2026-10-18 11:46:55 AEDT</t>
+          <t>2026-10-18 13:43:17 AEDT</t>
         </is>
       </c>
       <c r="AR5" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="AQ6" t="inlineStr">
         <is>
-          <t>2026-10-18 11:46:55 AEDT</t>
+          <t>2026-10-18 13:43:17 AEDT</t>
         </is>
       </c>
       <c r="AR6" t="inlineStr">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>2026-10-18 11:46:55 AEDT</t>
+          <t>2026-10-18 13:43:17 AEDT</t>
         </is>
       </c>
       <c r="AR7" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="AQ8" t="inlineStr">
         <is>
-          <t>2026-10-18 11:46:55 AEDT</t>
+          <t>2026-10-18 13:43:17 AEDT</t>
         </is>
       </c>
       <c r="AR8" t="inlineStr">
@@ -2730,7 +2730,7 @@
       </c>
       <c r="AQ9" t="inlineStr">
         <is>
-          <t>2026-10-18 11:46:55 AEDT</t>
+          <t>2026-10-18 13:43:17 AEDT</t>
         </is>
       </c>
       <c r="AR9" t="inlineStr">
@@ -2836,1590 +2836,6 @@
         </is>
       </c>
       <c r="BT9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>ALM</t>
-        </is>
-      </c>
-      <c r="B10" s="2">
-        <v>46325.375</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Brisbane Roar</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Auckland</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Previous</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Previous</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Previous</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>TEAM</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>previous-team fallback: TEAM is safer</t>
-        </is>
-      </c>
-      <c r="K10">
-        <v>3.261829908651272</v>
-      </c>
-      <c r="L10">
-        <v>3.484579853772908</v>
-      </c>
-      <c r="M10">
-        <v>2.460357622549616</v>
-      </c>
-      <c r="N10">
-        <v>3.261829908651272</v>
-      </c>
-      <c r="O10">
-        <v>3.484579853772908</v>
-      </c>
-      <c r="P10">
-        <v>2.460357622549616</v>
-      </c>
-      <c r="Q10">
-        <v>2.690253058706754</v>
-      </c>
-      <c r="R10">
-        <v>3.911525511001318</v>
-      </c>
-      <c r="S10">
-        <v>2.683605397121232</v>
-      </c>
-      <c r="T10">
-        <v>3.108172459895852</v>
-      </c>
-      <c r="U10">
-        <v>4.117911423114729</v>
-      </c>
-      <c r="V10">
-        <v>2.296601599291874</v>
-      </c>
-      <c r="W10">
-        <v>1.427834664843346</v>
-      </c>
-      <c r="X10">
-        <v>1.120414569680666</v>
-      </c>
-      <c r="Y10">
-        <v>2.548249234524013</v>
-      </c>
-      <c r="Z10">
-        <v>1.372091020195038</v>
-      </c>
-      <c r="AA10">
-        <v>1.37410388822717</v>
-      </c>
-      <c r="AB10">
-        <v>2.746194908422209</v>
-      </c>
-      <c r="AC10">
-        <v>1.349340690355546</v>
-      </c>
-      <c r="AD10">
-        <v>1.606811318152999</v>
-      </c>
-      <c r="AE10">
-        <v>2.956152008508545</v>
-      </c>
-      <c r="AF10">
-        <v>0.306576378292358</v>
-      </c>
-      <c r="AG10">
-        <v>0.2869786436138796</v>
-      </c>
-      <c r="AH10">
-        <v>0.4064449780937624</v>
-      </c>
-      <c r="AI10">
-        <v>-0.1999417413009712</v>
-      </c>
-      <c r="AJ10" t="inlineStr">
-        <is>
-          <t>Suncorp Stadium</t>
-        </is>
-      </c>
-      <c r="AK10" t="inlineStr">
-        <is>
-          <t>cross_country</t>
-        </is>
-      </c>
-      <c r="AL10">
-        <v>1.015664427141311</v>
-      </c>
-      <c r="AM10">
-        <v>1.215606168442283</v>
-      </c>
-      <c r="AN10" t="inlineStr">
-        <is>
-          <t>aleagues_team_player_joint_prod_v1.1.0</t>
-        </is>
-      </c>
-      <c r="AO10" t="inlineStr">
-        <is>
-          <t>ALM_2026/2027_wdw_0.99_none_l0.3_total_0.99_global_l0.3</t>
-        </is>
-      </c>
-      <c r="AP10" s="3">
-        <v>46165</v>
-      </c>
-      <c r="AQ10" t="inlineStr">
-        <is>
-          <t>2026-10-18 11:46:55 AEDT</t>
-        </is>
-      </c>
-      <c r="AR10" t="inlineStr">
-        <is>
-          <t>4ix8e8ynmhlhcnnbmfeu5xes4</t>
-        </is>
-      </c>
-      <c r="AS10" t="inlineStr">
-        <is>
-          <t>2026/2027</t>
-        </is>
-      </c>
-      <c r="AT10" t="inlineStr">
-        <is>
-          <t>Regular Season</t>
-        </is>
-      </c>
-      <c r="AU10" t="inlineStr">
-        <is>
-          <t>Fixture</t>
-        </is>
-      </c>
-      <c r="AV10" s="3">
-        <v>46325</v>
-      </c>
-      <c r="AW10" t="inlineStr">
-        <is>
-          <t>v046no35g7ebk8lytdjmfb43</t>
-        </is>
-      </c>
-      <c r="AX10" t="inlineStr">
-        <is>
-          <t>1csft77zeexrhddgjoxuht7v8</t>
-        </is>
-      </c>
-      <c r="AY10">
-        <v>0.3717122434871295</v>
-      </c>
-      <c r="AZ10">
-        <v>0.2556547304082412</v>
-      </c>
-      <c r="BA10">
-        <v>0.3726330261046293</v>
-      </c>
-      <c r="BB10">
-        <v>0.3217324691286621</v>
-      </c>
-      <c r="BC10">
-        <v>0.2428415517601431</v>
-      </c>
-      <c r="BD10">
-        <v>0.4354259791111948</v>
-      </c>
-      <c r="BE10">
-        <v>0.306576378292358</v>
-      </c>
-      <c r="BF10">
-        <v>0.2869786436138796</v>
-      </c>
-      <c r="BG10">
-        <v>0.4064449780937624</v>
-      </c>
-      <c r="BH10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BI10">
-        <v>0.8458305440641539</v>
-      </c>
-      <c r="BJ10">
-        <v>0.952947381716427</v>
-      </c>
-      <c r="BK10">
-        <v>1</v>
-      </c>
-      <c r="BL10">
-        <v>1</v>
-      </c>
-      <c r="BM10">
-        <v>0.4736924880542347</v>
-      </c>
-      <c r="BN10">
-        <v>0.3847484432182153</v>
-      </c>
-      <c r="BO10">
-        <v>0.06513586519477149</v>
-      </c>
-      <c r="BP10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BQ10" t="inlineStr">
-        <is>
-          <t>aleagues_player_signal_interval_hazard_v2.0.0</t>
-        </is>
-      </c>
-      <c r="BR10" t="inlineStr">
-        <is>
-          <t>aleagues_joint_player_poisson_box_prior_v1.2.0</t>
-        </is>
-      </c>
-      <c r="BS10" t="inlineStr">
-        <is>
-          <t>aleagues_binary_team_player_router_shadow_v1.0.0</t>
-        </is>
-      </c>
-      <c r="BT10" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>ALM</t>
-        </is>
-      </c>
-      <c r="B11" s="2">
-        <v>46326.16666666667</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Newcastle Jets</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Wellington Phoenix</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Previous</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Previous</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Previous</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>TEAM</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>previous-team fallback: TEAM is safer</t>
-        </is>
-      </c>
-      <c r="K11">
-        <v>2.63469117127551</v>
-      </c>
-      <c r="L11">
-        <v>3.611567385458002</v>
-      </c>
-      <c r="M11">
-        <v>2.910693098838093</v>
-      </c>
-      <c r="N11">
-        <v>2.63469117127551</v>
-      </c>
-      <c r="O11">
-        <v>3.611567385458002</v>
-      </c>
-      <c r="P11">
-        <v>2.910693098838093</v>
-      </c>
-      <c r="Q11">
-        <v>2.682636797954168</v>
-      </c>
-      <c r="R11">
-        <v>3.912646850621723</v>
-      </c>
-      <c r="S11">
-        <v>2.69069660542904</v>
-      </c>
-      <c r="T11">
-        <v>2.495739725886126</v>
-      </c>
-      <c r="U11">
-        <v>4.18849686564509</v>
-      </c>
-      <c r="V11">
-        <v>2.773401516373144</v>
-      </c>
-      <c r="W11">
-        <v>1.691565881891687</v>
-      </c>
-      <c r="X11">
-        <v>1.060871224028506</v>
-      </c>
-      <c r="Y11">
-        <v>2.752437105920193</v>
-      </c>
-      <c r="Z11">
-        <v>1.374997992233413</v>
-      </c>
-      <c r="AA11">
-        <v>1.372556523800535</v>
-      </c>
-      <c r="AB11">
-        <v>2.747554516033948</v>
-      </c>
-      <c r="AC11">
-        <v>1.590431463450688</v>
-      </c>
-      <c r="AD11">
-        <v>1.497999458609603</v>
-      </c>
-      <c r="AE11">
-        <v>3.088430922060291</v>
-      </c>
-      <c r="AF11">
-        <v>0.3795511257267692</v>
-      </c>
-      <c r="AG11">
-        <v>0.2768880913108547</v>
-      </c>
-      <c r="AH11">
-        <v>0.3435607829623761</v>
-      </c>
-      <c r="AI11">
-        <v>0.07411096730842415</v>
-      </c>
-      <c r="AJ11" t="inlineStr">
-        <is>
-          <t>McDonald Jones Stadium</t>
-        </is>
-      </c>
-      <c r="AK11" t="inlineStr">
-        <is>
-          <t>cross_country</t>
-        </is>
-      </c>
-      <c r="AL11">
-        <v>1.233358763047504</v>
-      </c>
-      <c r="AM11">
-        <v>1.15924779573908</v>
-      </c>
-      <c r="AN11" t="inlineStr">
-        <is>
-          <t>aleagues_team_player_joint_prod_v1.1.0</t>
-        </is>
-      </c>
-      <c r="AO11" t="inlineStr">
-        <is>
-          <t>ALM_2026/2027_wdw_0.99_none_l0.3_total_0.99_global_l0.3</t>
-        </is>
-      </c>
-      <c r="AP11" s="3">
-        <v>46165</v>
-      </c>
-      <c r="AQ11" t="inlineStr">
-        <is>
-          <t>2026-10-18 11:46:55 AEDT</t>
-        </is>
-      </c>
-      <c r="AR11" t="inlineStr">
-        <is>
-          <t>4ja4ia28n8xvxuec4o53kgsus</t>
-        </is>
-      </c>
-      <c r="AS11" t="inlineStr">
-        <is>
-          <t>2026/2027</t>
-        </is>
-      </c>
-      <c r="AT11" t="inlineStr">
-        <is>
-          <t>Regular Season</t>
-        </is>
-      </c>
-      <c r="AU11" t="inlineStr">
-        <is>
-          <t>Fixture</t>
-        </is>
-      </c>
-      <c r="AV11" s="3">
-        <v>46326</v>
-      </c>
-      <c r="AW11" t="inlineStr">
-        <is>
-          <t>chu9blh367xs3yumct5tqto2q</t>
-        </is>
-      </c>
-      <c r="AX11" t="inlineStr">
-        <is>
-          <t>6j4xzc2g1eeafo6v1f38d4x22</t>
-        </is>
-      </c>
-      <c r="AY11">
-        <v>0.3727675698635834</v>
-      </c>
-      <c r="AZ11">
-        <v>0.2555814613938641</v>
-      </c>
-      <c r="BA11">
-        <v>0.3716509687425524</v>
-      </c>
-      <c r="BB11">
-        <v>0.4006828074369593</v>
-      </c>
-      <c r="BC11">
-        <v>0.2387491341350175</v>
-      </c>
-      <c r="BD11">
-        <v>0.3605680584280232</v>
-      </c>
-      <c r="BE11">
-        <v>0.3795511257267692</v>
-      </c>
-      <c r="BF11">
-        <v>0.2768880913108547</v>
-      </c>
-      <c r="BG11">
-        <v>0.3435607829623761</v>
-      </c>
-      <c r="BH11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BI11">
-        <v>0.9060021598260801</v>
-      </c>
-      <c r="BJ11">
-        <v>0.8791943953205618</v>
-      </c>
-      <c r="BK11">
-        <v>1</v>
-      </c>
-      <c r="BL11">
-        <v>1</v>
-      </c>
-      <c r="BM11">
-        <v>0.3842705197258917</v>
-      </c>
-      <c r="BN11">
-        <v>0.4511831543178876</v>
-      </c>
-      <c r="BO11">
-        <v>0.0280901857801763</v>
-      </c>
-      <c r="BP11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BQ11" t="inlineStr">
-        <is>
-          <t>aleagues_player_signal_interval_hazard_v2.0.0</t>
-        </is>
-      </c>
-      <c r="BR11" t="inlineStr">
-        <is>
-          <t>aleagues_joint_player_poisson_box_prior_v1.2.0</t>
-        </is>
-      </c>
-      <c r="BS11" t="inlineStr">
-        <is>
-          <t>aleagues_binary_team_player_router_shadow_v1.0.0</t>
-        </is>
-      </c>
-      <c r="BT11" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>ALM</t>
-        </is>
-      </c>
-      <c r="B12" s="2">
-        <v>46326.25</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Melbourne City</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Sydney</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Previous</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Previous</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Previous</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>TEAM</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>previous-team fallback: TEAM is safer</t>
-        </is>
-      </c>
-      <c r="K12">
-        <v>2.700673681941764</v>
-      </c>
-      <c r="L12">
-        <v>3.538453796837892</v>
-      </c>
-      <c r="M12">
-        <v>2.880908671167313</v>
-      </c>
-      <c r="N12">
-        <v>2.700673681941764</v>
-      </c>
-      <c r="O12">
-        <v>3.538453796837892</v>
-      </c>
-      <c r="P12">
-        <v>2.880908671167313</v>
-      </c>
-      <c r="Q12">
-        <v>2.687051466177983</v>
-      </c>
-      <c r="R12">
-        <v>3.910353470606498</v>
-      </c>
-      <c r="S12">
-        <v>2.687352051925898</v>
-      </c>
-      <c r="T12">
-        <v>2.560804575724152</v>
-      </c>
-      <c r="U12">
-        <v>4.091576363505008</v>
-      </c>
-      <c r="V12">
-        <v>2.73902700826644</v>
-      </c>
-      <c r="W12">
-        <v>1.615458936296072</v>
-      </c>
-      <c r="X12">
-        <v>1.035928927995265</v>
-      </c>
-      <c r="Y12">
-        <v>2.651387864291338</v>
-      </c>
-      <c r="Z12">
-        <v>1.372433311542638</v>
-      </c>
-      <c r="AA12">
-        <v>1.372342335524878</v>
-      </c>
-      <c r="AB12">
-        <v>2.744775647067516</v>
-      </c>
-      <c r="AC12">
-        <v>1.512506369401032</v>
-      </c>
-      <c r="AD12">
-        <v>1.455008757612432</v>
-      </c>
-      <c r="AE12">
-        <v>2.967515127013464</v>
-      </c>
-      <c r="AF12">
-        <v>0.3702779816334595</v>
-      </c>
-      <c r="AG12">
-        <v>0.282609313959007</v>
-      </c>
-      <c r="AH12">
-        <v>0.3471127044075336</v>
-      </c>
-      <c r="AI12">
-        <v>0.04701328571641827</v>
-      </c>
-      <c r="AJ12" t="inlineStr">
-        <is>
-          <t>AAMI Park</t>
-        </is>
-      </c>
-      <c r="AK12" t="inlineStr">
-        <is>
-          <t>standard_home</t>
-        </is>
-      </c>
-      <c r="AL12">
-        <v>1.180241833529179</v>
-      </c>
-      <c r="AM12">
-        <v>1.133228547812761</v>
-      </c>
-      <c r="AN12" t="inlineStr">
-        <is>
-          <t>aleagues_team_player_joint_prod_v1.1.0</t>
-        </is>
-      </c>
-      <c r="AO12" t="inlineStr">
-        <is>
-          <t>ALM_2026/2027_wdw_0.99_none_l0.3_total_0.99_global_l0.3</t>
-        </is>
-      </c>
-      <c r="AP12" s="3">
-        <v>46165</v>
-      </c>
-      <c r="AQ12" t="inlineStr">
-        <is>
-          <t>2026-10-18 11:46:55 AEDT</t>
-        </is>
-      </c>
-      <c r="AR12" t="inlineStr">
-        <is>
-          <t>4jmx27tmmnrcndaplvfovqzo4</t>
-        </is>
-      </c>
-      <c r="AS12" t="inlineStr">
-        <is>
-          <t>2026/2027</t>
-        </is>
-      </c>
-      <c r="AT12" t="inlineStr">
-        <is>
-          <t>Regular Season</t>
-        </is>
-      </c>
-      <c r="AU12" t="inlineStr">
-        <is>
-          <t>Fixture</t>
-        </is>
-      </c>
-      <c r="AV12" s="3">
-        <v>46326</v>
-      </c>
-      <c r="AW12" t="inlineStr">
-        <is>
-          <t>c33jm806py6adse5wv9wx6ch1</t>
-        </is>
-      </c>
-      <c r="AX12" t="inlineStr">
-        <is>
-          <t>38ui5tfi8anjuh533emny2tz1</t>
-        </is>
-      </c>
-      <c r="AY12">
-        <v>0.3721551345729835</v>
-      </c>
-      <c r="AZ12">
-        <v>0.2557313571565436</v>
-      </c>
-      <c r="BA12">
-        <v>0.372113508270473</v>
-      </c>
-      <c r="BB12">
-        <v>0.3905022700598765</v>
-      </c>
-      <c r="BC12">
-        <v>0.2444045793497937</v>
-      </c>
-      <c r="BD12">
-        <v>0.3650931505903299</v>
-      </c>
-      <c r="BE12">
-        <v>0.3702779816334595</v>
-      </c>
-      <c r="BF12">
-        <v>0.282609313959007</v>
-      </c>
-      <c r="BG12">
-        <v>0.3471127044075336</v>
-      </c>
-      <c r="BH12" t="b">
-        <v>0</v>
-      </c>
-      <c r="BI12">
-        <v>0.7865844869915635</v>
-      </c>
-      <c r="BJ12">
-        <v>0.9632041759537114</v>
-      </c>
-      <c r="BK12">
-        <v>1</v>
-      </c>
-      <c r="BL12">
-        <v>1</v>
-      </c>
-      <c r="BM12">
-        <v>0.4670131761020158</v>
-      </c>
-      <c r="BN12">
-        <v>0.4273316030791136</v>
-      </c>
-      <c r="BO12">
-        <v>0.02687795680246335</v>
-      </c>
-      <c r="BP12" t="b">
-        <v>0</v>
-      </c>
-      <c r="BQ12" t="inlineStr">
-        <is>
-          <t>aleagues_player_signal_interval_hazard_v2.0.0</t>
-        </is>
-      </c>
-      <c r="BR12" t="inlineStr">
-        <is>
-          <t>aleagues_joint_player_poisson_box_prior_v1.2.0</t>
-        </is>
-      </c>
-      <c r="BS12" t="inlineStr">
-        <is>
-          <t>aleagues_binary_team_player_router_shadow_v1.0.0</t>
-        </is>
-      </c>
-      <c r="BT12" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>ALM</t>
-        </is>
-      </c>
-      <c r="B13" s="2">
-        <v>46326.36111111111</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Macarthur</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Western Sydney Wanderers</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Previous</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Previous</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Previous</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>TEAM</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>previous-team fallback: TEAM is safer</t>
-        </is>
-      </c>
-      <c r="K13">
-        <v>2.855198317270161</v>
-      </c>
-      <c r="L13">
-        <v>3.675867315882337</v>
-      </c>
-      <c r="M13">
-        <v>2.64748481452565</v>
-      </c>
-      <c r="N13">
-        <v>2.855198317270161</v>
-      </c>
-      <c r="O13">
-        <v>3.675867315882337</v>
-      </c>
-      <c r="P13">
-        <v>2.64748481452565</v>
-      </c>
-      <c r="Q13">
-        <v>2.684988279884119</v>
-      </c>
-      <c r="R13">
-        <v>3.913065498748149</v>
-      </c>
-      <c r="S13">
-        <v>2.688137514450082</v>
-      </c>
-      <c r="T13">
-        <v>2.721331780480031</v>
-      </c>
-      <c r="U13">
-        <v>4.259997297604807</v>
-      </c>
-      <c r="V13">
-        <v>2.513883364651093</v>
-      </c>
-      <c r="W13">
-        <v>1.658087735391341</v>
-      </c>
-      <c r="X13">
-        <v>1.148260713596349</v>
-      </c>
-      <c r="Y13">
-        <v>2.80634844898769</v>
-      </c>
-      <c r="Z13">
-        <v>1.374510133859729</v>
-      </c>
-      <c r="AA13">
-        <v>1.373556020948959</v>
-      </c>
-      <c r="AB13">
-        <v>2.748066154808688</v>
-      </c>
-      <c r="AC13">
-        <v>1.55704023427982</v>
-      </c>
-      <c r="AD13">
-        <v>1.627877089189346</v>
-      </c>
-      <c r="AE13">
-        <v>3.184917323469166</v>
-      </c>
-      <c r="AF13">
-        <v>0.350238368365282</v>
-      </c>
-      <c r="AG13">
-        <v>0.272044639826714</v>
-      </c>
-      <c r="AH13">
-        <v>0.377716991808004</v>
-      </c>
-      <c r="AI13">
-        <v>-0.05732667878017206</v>
-      </c>
-      <c r="AJ13" t="inlineStr">
-        <is>
-          <t>Campbelltown Sports Stadium</t>
-        </is>
-      </c>
-      <c r="AK13" t="inlineStr">
-        <is>
-          <t>same_city</t>
-        </is>
-      </c>
-      <c r="AL13">
-        <v>1.204701437858212</v>
-      </c>
-      <c r="AM13">
-        <v>1.262028116638384</v>
-      </c>
-      <c r="AN13" t="inlineStr">
-        <is>
-          <t>aleagues_team_player_joint_prod_v1.1.0</t>
-        </is>
-      </c>
-      <c r="AO13" t="inlineStr">
-        <is>
-          <t>ALM_2026/2027_wdw_0.99_none_l0.3_total_0.99_global_l0.3</t>
-        </is>
-      </c>
-      <c r="AP13" s="3">
-        <v>46165</v>
-      </c>
-      <c r="AQ13" t="inlineStr">
-        <is>
-          <t>2026-10-18 11:46:55 AEDT</t>
-        </is>
-      </c>
-      <c r="AR13" t="inlineStr">
-        <is>
-          <t>4jzsfga2fuu73vl1bg5vllmhg</t>
-        </is>
-      </c>
-      <c r="AS13" t="inlineStr">
-        <is>
-          <t>2026/2027</t>
-        </is>
-      </c>
-      <c r="AT13" t="inlineStr">
-        <is>
-          <t>Regular Season</t>
-        </is>
-      </c>
-      <c r="AU13" t="inlineStr">
-        <is>
-          <t>Fixture</t>
-        </is>
-      </c>
-      <c r="AV13" s="3">
-        <v>46326</v>
-      </c>
-      <c r="AW13" t="inlineStr">
-        <is>
-          <t>7jv344gvcvgqg7oeuc9u554dm</t>
-        </is>
-      </c>
-      <c r="AX13" t="inlineStr">
-        <is>
-          <t>6h553bwfqkoxayuv80uikkn42</t>
-        </is>
-      </c>
-      <c r="AY13">
-        <v>0.3724411043027565</v>
-      </c>
-      <c r="AZ13">
-        <v>0.2555541174355287</v>
-      </c>
-      <c r="BA13">
-        <v>0.3720047782617149</v>
-      </c>
-      <c r="BB13">
-        <v>0.3674671376614005</v>
-      </c>
-      <c r="BC13">
-        <v>0.2347419329496412</v>
-      </c>
-      <c r="BD13">
-        <v>0.3977909293889583</v>
-      </c>
-      <c r="BE13">
-        <v>0.350238368365282</v>
-      </c>
-      <c r="BF13">
-        <v>0.272044639826714</v>
-      </c>
-      <c r="BG13">
-        <v>0.377716991808004</v>
-      </c>
-      <c r="BH13" t="b">
-        <v>0</v>
-      </c>
-      <c r="BI13">
-        <v>0.8050226767240584</v>
-      </c>
-      <c r="BJ13">
-        <v>0.8297103291933792</v>
-      </c>
-      <c r="BK13">
-        <v>1</v>
-      </c>
-      <c r="BL13">
-        <v>1</v>
-      </c>
-      <c r="BM13">
-        <v>0.5123293552666615</v>
-      </c>
-      <c r="BN13">
-        <v>0.5212588960967434</v>
-      </c>
-      <c r="BO13">
-        <v>0.02220273593747446</v>
-      </c>
-      <c r="BP13" t="b">
-        <v>0</v>
-      </c>
-      <c r="BQ13" t="inlineStr">
-        <is>
-          <t>aleagues_player_signal_interval_hazard_v2.0.0</t>
-        </is>
-      </c>
-      <c r="BR13" t="inlineStr">
-        <is>
-          <t>aleagues_joint_player_poisson_box_prior_v1.2.0</t>
-        </is>
-      </c>
-      <c r="BS13" t="inlineStr">
-        <is>
-          <t>aleagues_binary_team_player_router_shadow_v1.0.0</t>
-        </is>
-      </c>
-      <c r="BT13" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>ALM</t>
-        </is>
-      </c>
-      <c r="B14" s="2">
-        <v>46327.16666666667</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Melbourne Victory</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Central Coast Mariners</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Previous</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Previous</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Previous</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>TEAM</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>previous-team fallback: TEAM is safer</t>
-        </is>
-      </c>
-      <c r="K14">
-        <v>2.688489409188326</v>
-      </c>
-      <c r="L14">
-        <v>3.540237439612302</v>
-      </c>
-      <c r="M14">
-        <v>2.893711235751404</v>
-      </c>
-      <c r="N14">
-        <v>2.688489409188326</v>
-      </c>
-      <c r="O14">
-        <v>3.540237439612302</v>
-      </c>
-      <c r="P14">
-        <v>2.893711235751404</v>
-      </c>
-      <c r="Q14">
-        <v>2.683967800445223</v>
-      </c>
-      <c r="R14">
-        <v>3.912468506103089</v>
-      </c>
-      <c r="S14">
-        <v>2.689443187914418</v>
-      </c>
-      <c r="T14">
-        <v>2.545310871139171</v>
-      </c>
-      <c r="U14">
-        <v>4.100820062473706</v>
-      </c>
-      <c r="V14">
-        <v>2.752796023180379</v>
-      </c>
-      <c r="W14">
-        <v>1.626682425375765</v>
-      </c>
-      <c r="X14">
-        <v>1.032505813205105</v>
-      </c>
-      <c r="Y14">
-        <v>2.65918823858087</v>
-      </c>
-      <c r="Z14">
-        <v>1.374499361960165</v>
-      </c>
-      <c r="AA14">
-        <v>1.372840870517284</v>
-      </c>
-      <c r="AB14">
-        <v>2.747340232477448</v>
-      </c>
-      <c r="AC14">
-        <v>1.522773488578821</v>
-      </c>
-      <c r="AD14">
-        <v>1.455651496165577</v>
-      </c>
-      <c r="AE14">
-        <v>2.978424984744398</v>
-      </c>
-      <c r="AF14">
-        <v>0.3719560867832866</v>
-      </c>
-      <c r="AG14">
-        <v>0.2824669297067012</v>
-      </c>
-      <c r="AH14">
-        <v>0.3455769835100122</v>
-      </c>
-      <c r="AI14">
-        <v>0.05355256196532188</v>
-      </c>
-      <c r="AJ14" t="inlineStr">
-        <is>
-          <t>AAMI Park</t>
-        </is>
-      </c>
-      <c r="AK14" t="inlineStr">
-        <is>
-          <t>standard_home</t>
-        </is>
-      </c>
-      <c r="AL14">
-        <v>1.18428733971099</v>
-      </c>
-      <c r="AM14">
-        <v>1.130734777745668</v>
-      </c>
-      <c r="AN14" t="inlineStr">
-        <is>
-          <t>aleagues_team_player_joint_prod_v1.1.0</t>
-        </is>
-      </c>
-      <c r="AO14" t="inlineStr">
-        <is>
-          <t>ALM_2026/2027_wdw_0.99_none_l0.3_total_0.99_global_l0.3</t>
-        </is>
-      </c>
-      <c r="AP14" s="3">
-        <v>46165</v>
-      </c>
-      <c r="AQ14" t="inlineStr">
-        <is>
-          <t>2026-10-18 11:46:55 AEDT</t>
-        </is>
-      </c>
-      <c r="AR14" t="inlineStr">
-        <is>
-          <t>4kcl9ql01ij96lr9st00k5jis</t>
-        </is>
-      </c>
-      <c r="AS14" t="inlineStr">
-        <is>
-          <t>2026/2027</t>
-        </is>
-      </c>
-      <c r="AT14" t="inlineStr">
-        <is>
-          <t>Regular Season</t>
-        </is>
-      </c>
-      <c r="AU14" t="inlineStr">
-        <is>
-          <t>Fixture</t>
-        </is>
-      </c>
-      <c r="AV14" s="3">
-        <v>46327</v>
-      </c>
-      <c r="AW14" t="inlineStr">
-        <is>
-          <t>9xmhnv6im8h7c9e17oqvcx8gl</t>
-        </is>
-      </c>
-      <c r="AX14" t="inlineStr">
-        <is>
-          <t>c4ygb6mnh53kpl2mpxe52l8jw</t>
-        </is>
-      </c>
-      <c r="AY14">
-        <v>0.3725827112509015</v>
-      </c>
-      <c r="AZ14">
-        <v>0.255593111724757</v>
-      </c>
-      <c r="BA14">
-        <v>0.3718241770243415</v>
-      </c>
-      <c r="BB14">
-        <v>0.3928793183334982</v>
-      </c>
-      <c r="BC14">
-        <v>0.2438536645757575</v>
-      </c>
-      <c r="BD14">
-        <v>0.3632670170907444</v>
-      </c>
-      <c r="BE14">
-        <v>0.3719560867832866</v>
-      </c>
-      <c r="BF14">
-        <v>0.2824669297067012</v>
-      </c>
-      <c r="BG14">
-        <v>0.3455769835100122</v>
-      </c>
-      <c r="BH14" t="b">
-        <v>0</v>
-      </c>
-      <c r="BI14">
-        <v>0.8878408610668614</v>
-      </c>
-      <c r="BJ14">
-        <v>0.9055908690094202</v>
-      </c>
-      <c r="BK14">
-        <v>1</v>
-      </c>
-      <c r="BL14">
-        <v>1</v>
-      </c>
-      <c r="BM14">
-        <v>0.4390459306002075</v>
-      </c>
-      <c r="BN14">
-        <v>0.4751833483035187</v>
-      </c>
-      <c r="BO14">
-        <v>0.02687381798194416</v>
-      </c>
-      <c r="BP14" t="b">
-        <v>0</v>
-      </c>
-      <c r="BQ14" t="inlineStr">
-        <is>
-          <t>aleagues_player_signal_interval_hazard_v2.0.0</t>
-        </is>
-      </c>
-      <c r="BR14" t="inlineStr">
-        <is>
-          <t>aleagues_joint_player_poisson_box_prior_v1.2.0</t>
-        </is>
-      </c>
-      <c r="BS14" t="inlineStr">
-        <is>
-          <t>aleagues_binary_team_player_router_shadow_v1.0.0</t>
-        </is>
-      </c>
-      <c r="BT14" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>ALM</t>
-        </is>
-      </c>
-      <c r="B15" s="2">
-        <v>46327.33333333333</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Perth Glory</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Adelaide United</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Previous</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Previous</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Previous</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>TEAM</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>previous-team fallback: TEAM is safer</t>
-        </is>
-      </c>
-      <c r="K15">
-        <v>3.082152621894857</v>
-      </c>
-      <c r="L15">
-        <v>3.786861796274146</v>
-      </c>
-      <c r="M15">
-        <v>2.430248619108524</v>
-      </c>
-      <c r="N15">
-        <v>3.082152621894857</v>
-      </c>
-      <c r="O15">
-        <v>3.786861796274146</v>
-      </c>
-      <c r="P15">
-        <v>2.430248619108524</v>
-      </c>
-      <c r="Q15">
-        <v>2.687507681707328</v>
-      </c>
-      <c r="R15">
-        <v>3.912345690684275</v>
-      </c>
-      <c r="S15">
-        <v>2.685956092730187</v>
-      </c>
-      <c r="T15">
-        <v>2.959151301166934</v>
-      </c>
-      <c r="U15">
-        <v>4.379303043300208</v>
-      </c>
-      <c r="V15">
-        <v>2.30564331138719</v>
-      </c>
-      <c r="W15">
-        <v>1.641712211078597</v>
-      </c>
-      <c r="X15">
-        <v>1.24875379713097</v>
-      </c>
-      <c r="Y15">
-        <v>2.890466008209566</v>
-      </c>
-      <c r="Z15">
-        <v>1.373361468450402</v>
-      </c>
-      <c r="AA15">
-        <v>1.373831422931391</v>
-      </c>
-      <c r="AB15">
-        <v>2.747192891381793</v>
-      </c>
-      <c r="AC15">
-        <v>1.541136491509765</v>
-      </c>
-      <c r="AD15">
-        <v>1.769225243624263</v>
-      </c>
-      <c r="AE15">
-        <v>3.310361735134028</v>
-      </c>
-      <c r="AF15">
-        <v>0.3244485665298483</v>
-      </c>
-      <c r="AG15">
-        <v>0.2640708992823265</v>
-      </c>
-      <c r="AH15">
-        <v>0.4114805341878253</v>
-      </c>
-      <c r="AI15">
-        <v>-0.1852171886290896</v>
-      </c>
-      <c r="AJ15" t="inlineStr">
-        <is>
-          <t>HBF Park</t>
-        </is>
-      </c>
-      <c r="AK15" t="inlineStr">
-        <is>
-          <t>standard_home</t>
-        </is>
-      </c>
-      <c r="AL15">
-        <v>1.194665556086594</v>
-      </c>
-      <c r="AM15">
-        <v>1.379882744715684</v>
-      </c>
-      <c r="AN15" t="inlineStr">
-        <is>
-          <t>aleagues_team_player_joint_prod_v1.1.0</t>
-        </is>
-      </c>
-      <c r="AO15" t="inlineStr">
-        <is>
-          <t>ALM_2026/2027_wdw_0.99_none_l0.3_total_0.99_global_l0.3</t>
-        </is>
-      </c>
-      <c r="AP15" s="3">
-        <v>46165</v>
-      </c>
-      <c r="AQ15" t="inlineStr">
-        <is>
-          <t>2026-10-18 11:46:55 AEDT</t>
-        </is>
-      </c>
-      <c r="AR15" t="inlineStr">
-        <is>
-          <t>4kq69vmye8oqugawrbux6il90</t>
-        </is>
-      </c>
-      <c r="AS15" t="inlineStr">
-        <is>
-          <t>2026/2027</t>
-        </is>
-      </c>
-      <c r="AT15" t="inlineStr">
-        <is>
-          <t>Regular Season</t>
-        </is>
-      </c>
-      <c r="AU15" t="inlineStr">
-        <is>
-          <t>Fixture</t>
-        </is>
-      </c>
-      <c r="AV15" s="3">
-        <v>46327</v>
-      </c>
-      <c r="AW15" t="inlineStr">
-        <is>
-          <t>cuj4qahgk4idsme4dg8clk6gw</t>
-        </is>
-      </c>
-      <c r="AX15" t="inlineStr">
-        <is>
-          <t>6lezh5aazy0xca1800e5dqxwl</t>
-        </is>
-      </c>
-      <c r="AY15">
-        <v>0.372091959701755</v>
-      </c>
-      <c r="AZ15">
-        <v>0.2556011352424991</v>
-      </c>
-      <c r="BA15">
-        <v>0.3723069050557459</v>
-      </c>
-      <c r="BB15">
-        <v>0.3379347313554574</v>
-      </c>
-      <c r="BC15">
-        <v>0.2283468374105501</v>
-      </c>
-      <c r="BD15">
-        <v>0.4337184312339926</v>
-      </c>
-      <c r="BE15">
-        <v>0.3244485665298483</v>
-      </c>
-      <c r="BF15">
-        <v>0.2640708992823265</v>
-      </c>
-      <c r="BG15">
-        <v>0.4114805341878253</v>
-      </c>
-      <c r="BH15" t="b">
-        <v>0</v>
-      </c>
-      <c r="BI15">
-        <v>0.9560816341569174</v>
-      </c>
-      <c r="BJ15">
-        <v>0.8900358093794883</v>
-      </c>
-      <c r="BK15">
-        <v>1</v>
-      </c>
-      <c r="BL15">
-        <v>1</v>
-      </c>
-      <c r="BM15">
-        <v>0.4410532645932226</v>
-      </c>
-      <c r="BN15">
-        <v>0.4060941615544638</v>
-      </c>
-      <c r="BO15">
-        <v>0.04764339317190669</v>
-      </c>
-      <c r="BP15" t="b">
-        <v>0</v>
-      </c>
-      <c r="BQ15" t="inlineStr">
-        <is>
-          <t>aleagues_player_signal_interval_hazard_v2.0.0</t>
-        </is>
-      </c>
-      <c r="BR15" t="inlineStr">
-        <is>
-          <t>aleagues_joint_player_poisson_box_prior_v1.2.0</t>
-        </is>
-      </c>
-      <c r="BS15" t="inlineStr">
-        <is>
-          <t>aleagues_binary_team_player_router_shadow_v1.0.0</t>
-        </is>
-      </c>
-      <c r="BT15" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update model outputs 2026-10-20 17:50:08
</commit_message>
<xml_diff>
--- a/files/A-Leagues_upcoming_projections.xlsx
+++ b/files/A-Leagues_upcoming_projections.xlsx
@@ -882,7 +882,7 @@
       </c>
       <c r="AQ2" t="inlineStr">
         <is>
-          <t>2026-10-18 13:43:17 AEDT</t>
+          <t>2026-10-19 17:23:56 AEDT</t>
         </is>
       </c>
       <c r="AR2" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="AQ3" t="inlineStr">
         <is>
-          <t>2026-10-18 13:43:17 AEDT</t>
+          <t>2026-10-19 17:23:56 AEDT</t>
         </is>
       </c>
       <c r="AR3" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="AQ4" t="inlineStr">
         <is>
-          <t>2026-10-18 13:43:17 AEDT</t>
+          <t>2026-10-19 17:23:56 AEDT</t>
         </is>
       </c>
       <c r="AR4" t="inlineStr">
@@ -1674,7 +1674,7 @@
       </c>
       <c r="AQ5" t="inlineStr">
         <is>
-          <t>2026-10-18 13:43:17 AEDT</t>
+          <t>2026-10-19 17:23:56 AEDT</t>
         </is>
       </c>
       <c r="AR5" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="AQ6" t="inlineStr">
         <is>
-          <t>2026-10-18 13:43:17 AEDT</t>
+          <t>2026-10-19 17:23:56 AEDT</t>
         </is>
       </c>
       <c r="AR6" t="inlineStr">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>2026-10-18 13:43:17 AEDT</t>
+          <t>2026-10-19 17:23:56 AEDT</t>
         </is>
       </c>
       <c r="AR7" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="AQ8" t="inlineStr">
         <is>
-          <t>2026-10-18 13:43:17 AEDT</t>
+          <t>2026-10-19 17:23:56 AEDT</t>
         </is>
       </c>
       <c r="AR8" t="inlineStr">
@@ -2730,7 +2730,7 @@
       </c>
       <c r="AQ9" t="inlineStr">
         <is>
-          <t>2026-10-18 13:43:17 AEDT</t>
+          <t>2026-10-19 17:23:56 AEDT</t>
         </is>
       </c>
       <c r="AR9" t="inlineStr">

</xml_diff>

<commit_message>
Update model outputs 2026-10-21 22:24:42
</commit_message>
<xml_diff>
--- a/files/A-Leagues_upcoming_projections.xlsx
+++ b/files/A-Leagues_upcoming_projections.xlsx
@@ -882,7 +882,7 @@
       </c>
       <c r="AQ2" t="inlineStr">
         <is>
-          <t>2026-10-19 17:23:56 AEDT</t>
+          <t>2026-10-21 15:31:13 AEDT</t>
         </is>
       </c>
       <c r="AR2" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="AQ3" t="inlineStr">
         <is>
-          <t>2026-10-19 17:23:56 AEDT</t>
+          <t>2026-10-21 15:31:13 AEDT</t>
         </is>
       </c>
       <c r="AR3" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="AQ4" t="inlineStr">
         <is>
-          <t>2026-10-19 17:23:56 AEDT</t>
+          <t>2026-10-21 15:31:13 AEDT</t>
         </is>
       </c>
       <c r="AR4" t="inlineStr">
@@ -1674,7 +1674,7 @@
       </c>
       <c r="AQ5" t="inlineStr">
         <is>
-          <t>2026-10-19 17:23:56 AEDT</t>
+          <t>2026-10-21 15:31:13 AEDT</t>
         </is>
       </c>
       <c r="AR5" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="AQ6" t="inlineStr">
         <is>
-          <t>2026-10-19 17:23:56 AEDT</t>
+          <t>2026-10-21 15:31:13 AEDT</t>
         </is>
       </c>
       <c r="AR6" t="inlineStr">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>2026-10-19 17:23:56 AEDT</t>
+          <t>2026-10-21 15:31:13 AEDT</t>
         </is>
       </c>
       <c r="AR7" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="AQ8" t="inlineStr">
         <is>
-          <t>2026-10-19 17:23:56 AEDT</t>
+          <t>2026-10-21 15:31:13 AEDT</t>
         </is>
       </c>
       <c r="AR8" t="inlineStr">
@@ -2730,7 +2730,7 @@
       </c>
       <c r="AQ9" t="inlineStr">
         <is>
-          <t>2026-10-19 17:23:56 AEDT</t>
+          <t>2026-10-21 15:31:13 AEDT</t>
         </is>
       </c>
       <c r="AR9" t="inlineStr">

</xml_diff>

<commit_message>
Update model outputs 2026-10-22 22:41:47
</commit_message>
<xml_diff>
--- a/files/A-Leagues_upcoming_projections.xlsx
+++ b/files/A-Leagues_upcoming_projections.xlsx
@@ -357,7 +357,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BT9"/>
+  <dimension ref="A1:BT12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -734,21 +734,21 @@
         </is>
       </c>
       <c r="B2" s="2">
-        <v>46313.08333333333</v>
+        <v>46318.375</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Wellington Phoenix</t>
+          <t>Brisbane Roar</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Melbourne Victory</t>
+          <t>Perth Glory</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -777,95 +777,95 @@
         </is>
       </c>
       <c r="K2">
-        <v>3.044882281541064</v>
+        <v>2.68252353918019</v>
       </c>
       <c r="L2">
-        <v>3.51574201897158</v>
+        <v>3.581857690447499</v>
       </c>
       <c r="M2">
-        <v>2.583010855628705</v>
+        <v>2.873299388701397</v>
       </c>
       <c r="N2">
-        <v>3.044882281541064</v>
+        <v>2.68252353918019</v>
       </c>
       <c r="O2">
-        <v>3.51574201897158</v>
+        <v>3.581857690447499</v>
       </c>
       <c r="P2">
-        <v>2.583010855628705</v>
+        <v>2.873299388701397</v>
       </c>
       <c r="Q2">
-        <v>2.689919199858007</v>
+        <v>2.698163403448263</v>
       </c>
       <c r="R2">
-        <v>3.912374862151778</v>
+        <v>3.868048822711331</v>
       </c>
       <c r="S2">
-        <v>2.683537947480759</v>
+        <v>2.696513498687903</v>
       </c>
       <c r="T2">
-        <v>2.900364107659429</v>
+        <v>2.54184513739414</v>
       </c>
       <c r="U2">
-        <v>4.080318680837341</v>
+        <v>4.161147462249319</v>
       </c>
       <c r="V2">
-        <v>2.438210822416481</v>
+        <v>2.730251128252911</v>
       </c>
       <c r="W2">
-        <v>1.495211940925515</v>
+        <v>1.661832212476893</v>
       </c>
       <c r="X2">
-        <v>1.091950292634631</v>
+        <v>1.058294745427542</v>
       </c>
       <c r="Y2">
-        <v>2.587162233560146</v>
+        <v>2.720126957904435</v>
       </c>
       <c r="Z2">
-        <v>1.372646545137794</v>
+        <v>1.34662291166073</v>
       </c>
       <c r="AA2">
-        <v>1.374579354599392</v>
+        <v>1.347114450087493</v>
       </c>
       <c r="AB2">
-        <v>2.747225899737185</v>
+        <v>2.693737361748223</v>
       </c>
       <c r="AC2">
-        <v>1.39641660097865</v>
+        <v>1.55927565645795</v>
       </c>
       <c r="AD2">
-        <v>1.543799335084466</v>
+        <v>1.497024921290691</v>
       </c>
       <c r="AE2">
-        <v>2.940215936063116</v>
+        <v>3.05630057774864</v>
       </c>
       <c r="AF2">
-        <v>0.3284199215392603</v>
+        <v>0.3727833084758733</v>
       </c>
       <c r="AG2">
-        <v>0.2844349769134991</v>
+        <v>0.2791847377596582</v>
       </c>
       <c r="AH2">
-        <v>0.3871451015472407</v>
+        <v>0.3480319537644685</v>
       </c>
       <c r="AI2">
-        <v>-0.1185347701922317</v>
+        <v>0.05067388586567256</v>
       </c>
       <c r="AJ2" t="inlineStr">
         <is>
-          <t>Hnry Stadium</t>
+          <t>Suncorp Stadium</t>
         </is>
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>cross_country</t>
+          <t>standard_home</t>
         </is>
       </c>
       <c r="AL2">
-        <v>1.081325349881739</v>
+        <v>1.205975929186521</v>
       </c>
       <c r="AM2">
-        <v>1.19986012007397</v>
+        <v>1.155302043320848</v>
       </c>
       <c r="AN2" t="inlineStr">
         <is>
@@ -878,16 +878,16 @@
         </is>
       </c>
       <c r="AP2" s="3">
-        <v>46165</v>
+        <v>46313</v>
       </c>
       <c r="AQ2" t="inlineStr">
         <is>
-          <t>2026-10-21 15:31:13 AEDT</t>
+          <t>2026-10-22 21:56:26 AEDT</t>
         </is>
       </c>
       <c r="AR2" t="inlineStr">
         <is>
-          <t>4fvv54cadlavkl7k6twdfoy6s</t>
+          <t>4gpo8d0qh5hhucerumdq73dhw</t>
         </is>
       </c>
       <c r="AS2" t="inlineStr">
@@ -906,53 +906,53 @@
         </is>
       </c>
       <c r="AV2" s="3">
-        <v>46313</v>
+        <v>46318</v>
       </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>6j4xzc2g1eeafo6v1f38d4x22</t>
+          <t>v046no35g7ebk8lytdjmfb43</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>9xmhnv6im8h7c9e17oqvcx8gl</t>
+          <t>cuj4qahgk4idsme4dg8clk6gw</t>
         </is>
       </c>
       <c r="AY2">
-        <v>0.3717583784869029</v>
+        <v>0.3706224755409536</v>
       </c>
       <c r="AZ2">
-        <v>0.2555992294281349</v>
+        <v>0.2585282776495681</v>
       </c>
       <c r="BA2">
-        <v>0.3726423920849622</v>
+        <v>0.3708492468094783</v>
       </c>
       <c r="BB2">
-        <v>0.3447842970333101</v>
+        <v>0.3934149981399672</v>
       </c>
       <c r="BC2">
-        <v>0.2450788965813781</v>
+        <v>0.2403183278343727</v>
       </c>
       <c r="BD2">
-        <v>0.4101368063853117</v>
+        <v>0.3662666740256602</v>
       </c>
       <c r="BE2">
-        <v>0.3284199215392603</v>
+        <v>0.3727833084758733</v>
       </c>
       <c r="BF2">
-        <v>0.2844349769134991</v>
+        <v>0.2791847377596582</v>
       </c>
       <c r="BG2">
-        <v>0.3871451015472407</v>
+        <v>0.3480319537644685</v>
       </c>
       <c r="BH2" t="b">
         <v>0</v>
       </c>
       <c r="BI2">
-        <v>0.8791943953205618</v>
+        <v>0.8458305440641539</v>
       </c>
       <c r="BJ2">
-        <v>0.8878408610668614</v>
+        <v>0.9560816341569174</v>
       </c>
       <c r="BK2">
         <v>1</v>
@@ -961,13 +961,13 @@
         <v>1</v>
       </c>
       <c r="BM2">
-        <v>0.4511831543178876</v>
+        <v>0.4736924880542347</v>
       </c>
       <c r="BN2">
-        <v>0.4390459306002075</v>
+        <v>0.4410532645932226</v>
       </c>
       <c r="BO2">
-        <v>0.04333845694764266</v>
+        <v>0.02281729304500985</v>
       </c>
       <c r="BP2" t="b">
         <v>0</v>
@@ -998,21 +998,21 @@
         </is>
       </c>
       <c r="B3" s="2">
-        <v>46313.16666666667</v>
+        <v>46319.16666666667</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Adelaide United</t>
+          <t>Newcastle Jets</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Brisbane Roar</t>
+          <t>Macarthur</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1041,83 +1041,83 @@
         </is>
       </c>
       <c r="K3">
-        <v>2.529078068707507</v>
+        <v>2.627885640906318</v>
       </c>
       <c r="L3">
-        <v>3.69920729247915</v>
+        <v>3.709527375301805</v>
       </c>
       <c r="M3">
-        <v>2.99158635320507</v>
+        <v>2.85804260024231</v>
       </c>
       <c r="N3">
-        <v>2.529078068707507</v>
+        <v>2.627885640906318</v>
       </c>
       <c r="O3">
-        <v>3.69920729247915</v>
+        <v>3.709527375301805</v>
       </c>
       <c r="P3">
-        <v>2.99158635320507</v>
+        <v>2.85804260024231</v>
       </c>
       <c r="Q3">
-        <v>2.685095842341116</v>
+        <v>2.69422727168237</v>
       </c>
       <c r="R3">
-        <v>3.912487510869863</v>
+        <v>3.869244114220696</v>
       </c>
       <c r="S3">
-        <v>2.688302518522552</v>
+        <v>2.699874032213838</v>
       </c>
       <c r="T3">
-        <v>2.397673111172344</v>
+        <v>2.496129166976444</v>
       </c>
       <c r="U3">
-        <v>4.282638857730398</v>
+        <v>4.293538884263335</v>
       </c>
       <c r="V3">
-        <v>2.861819282537725</v>
+        <v>2.728724389863987</v>
       </c>
       <c r="W3">
-        <v>1.788611734944091</v>
+        <v>1.765427456689718</v>
       </c>
       <c r="X3">
-        <v>1.07520475259988</v>
+        <v>1.110051131746342</v>
       </c>
       <c r="Y3">
-        <v>2.863816487543971</v>
+        <v>2.87547858843606</v>
       </c>
       <c r="Z3">
-        <v>1.37416792035036</v>
+        <v>1.348426490703327</v>
       </c>
       <c r="AA3">
-        <v>1.373196612518503</v>
+        <v>1.346743457629564</v>
       </c>
       <c r="AB3">
-        <v>2.747364532868863</v>
+        <v>2.695169948332891</v>
       </c>
       <c r="AC3">
-        <v>1.679379355538903</v>
+        <v>1.654395724314069</v>
       </c>
       <c r="AD3">
-        <v>1.520901724625932</v>
+        <v>1.574128104772371</v>
       </c>
       <c r="AE3">
-        <v>3.200281080164835</v>
+        <v>3.22852382908644</v>
       </c>
       <c r="AF3">
-        <v>0.3954010010102429</v>
+        <v>0.3805340629872749</v>
       </c>
       <c r="AG3">
-        <v>0.2703281868072378</v>
+        <v>0.2695761208444083</v>
       </c>
       <c r="AH3">
-        <v>0.3342708121825193</v>
+        <v>0.3498898161683168</v>
       </c>
       <c r="AI3">
-        <v>0.1280102472688327</v>
+        <v>0.0643577185172497</v>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>Coopers Stadium</t>
+          <t>McDonald Jones Stadium</t>
         </is>
       </c>
       <c r="AK3" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="AL3">
-        <v>1.3064555955987</v>
+        <v>1.28454341492864</v>
       </c>
       <c r="AM3">
-        <v>1.178445348329868</v>
+        <v>1.22018569641139</v>
       </c>
       <c r="AN3" t="inlineStr">
         <is>
@@ -1142,16 +1142,16 @@
         </is>
       </c>
       <c r="AP3" s="3">
-        <v>46165</v>
+        <v>46313</v>
       </c>
       <c r="AQ3" t="inlineStr">
         <is>
-          <t>2026-10-21 15:31:13 AEDT</t>
+          <t>2026-10-22 21:56:26 AEDT</t>
         </is>
       </c>
       <c r="AR3" t="inlineStr">
         <is>
-          <t>4gc631hxb8kjwe3gs3o2rblsk</t>
+          <t>4h3a60ofbfqccw27euzi80qhg</t>
         </is>
       </c>
       <c r="AS3" t="inlineStr">
@@ -1170,53 +1170,53 @@
         </is>
       </c>
       <c r="AV3" s="3">
-        <v>46313</v>
+        <v>46319</v>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>6lezh5aazy0xca1800e5dqxwl</t>
+          <t>chu9blh367xs3yumct5tqto2q</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr">
         <is>
-          <t>v046no35g7ebk8lytdjmfb43</t>
+          <t>7jv344gvcvgqg7oeuc9u554dm</t>
         </is>
       </c>
       <c r="AY3">
-        <v>0.3724261846564504</v>
+        <v>0.3711639365062046</v>
       </c>
       <c r="AZ3">
-        <v>0.2555918701904482</v>
+        <v>0.258448412785506</v>
       </c>
       <c r="BA3">
-        <v>0.3719819451531013</v>
+        <v>0.3703876507082894</v>
       </c>
       <c r="BB3">
-        <v>0.4170710324690797</v>
+        <v>0.4006202937051122</v>
       </c>
       <c r="BC3">
-        <v>0.2335008935425281</v>
+        <v>0.232908103770807</v>
       </c>
       <c r="BD3">
-        <v>0.3494280739883923</v>
+        <v>0.3664716025240808</v>
       </c>
       <c r="BE3">
-        <v>0.3954010010102429</v>
+        <v>0.3805340629872749</v>
       </c>
       <c r="BF3">
-        <v>0.2703281868072378</v>
+        <v>0.2695761208444083</v>
       </c>
       <c r="BG3">
-        <v>0.3342708121825193</v>
+        <v>0.3498898161683168</v>
       </c>
       <c r="BH3" t="b">
         <v>0</v>
       </c>
       <c r="BI3">
-        <v>0.8900358093794883</v>
+        <v>0.9060021598260801</v>
       </c>
       <c r="BJ3">
-        <v>0.8458305440641539</v>
+        <v>0.8050226767240584</v>
       </c>
       <c r="BK3">
         <v>1</v>
@@ -1225,13 +1225,13 @@
         <v>1</v>
       </c>
       <c r="BM3">
-        <v>0.4060941615544638</v>
+        <v>0.3842705197258917</v>
       </c>
       <c r="BN3">
-        <v>0.4736924880542347</v>
+        <v>0.5123293552666615</v>
       </c>
       <c r="BO3">
-        <v>0.03771113297058198</v>
+        <v>0.02049783453997267</v>
       </c>
       <c r="BP3" t="b">
         <v>0</v>
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <v>46318.375</v>
+        <v>46319.25</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -1271,12 +1271,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Brisbane Roar</t>
+          <t>Western Sydney Wanderers</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Perth Glory</t>
+          <t>Auckland</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1305,95 +1305,95 @@
         </is>
       </c>
       <c r="K4">
-        <v>2.686218715277394</v>
+        <v>3.013953531406892</v>
       </c>
       <c r="L4">
-        <v>3.582785987704285</v>
+        <v>3.518756051443509</v>
       </c>
       <c r="M4">
-        <v>2.868476676142175</v>
+        <v>2.604040936654958</v>
       </c>
       <c r="N4">
-        <v>2.686218715277394</v>
+        <v>3.013953531406892</v>
       </c>
       <c r="O4">
-        <v>3.582785987704285</v>
+        <v>3.518756051443509</v>
       </c>
       <c r="P4">
-        <v>2.868476676142175</v>
+        <v>2.604040936654958</v>
       </c>
       <c r="Q4">
-        <v>2.687645390717474</v>
+        <v>2.701394919900912</v>
       </c>
       <c r="R4">
-        <v>3.911981160795712</v>
+        <v>3.867828504560829</v>
       </c>
       <c r="S4">
-        <v>2.685990379374191</v>
+        <v>2.693400469127965</v>
       </c>
       <c r="T4">
-        <v>2.545602539861762</v>
+        <v>2.863417991757246</v>
       </c>
       <c r="U4">
-        <v>4.162143364080644</v>
+        <v>4.14228256736555</v>
       </c>
       <c r="V4">
-        <v>2.725502106741051</v>
+        <v>2.442872048678385</v>
       </c>
       <c r="W4">
-        <v>1.659223168266833</v>
+        <v>1.530929954448405</v>
       </c>
       <c r="X4">
-        <v>1.059345277299219</v>
+        <v>1.099898803120357</v>
       </c>
       <c r="Y4">
-        <v>2.718568445566051</v>
+        <v>2.630828757568762</v>
       </c>
       <c r="Z4">
-        <v>1.373124619550372</v>
+        <v>1.345543931909936</v>
       </c>
       <c r="AA4">
-        <v>1.373625831515056</v>
+        <v>1.34792542963059</v>
       </c>
       <c r="AB4">
-        <v>2.746750451065429</v>
+        <v>2.693469361540526</v>
       </c>
       <c r="AC4">
-        <v>1.558649997387424</v>
+        <v>1.442020749634317</v>
       </c>
       <c r="AD4">
-        <v>1.499181579965792</v>
+        <v>1.579246941817202</v>
       </c>
       <c r="AE4">
-        <v>3.057831577353215</v>
+        <v>3.021267691451519</v>
       </c>
       <c r="AF4">
-        <v>0.3722705058648712</v>
+        <v>0.3317901187193179</v>
       </c>
       <c r="AG4">
-        <v>0.2791124011961325</v>
+        <v>0.2841913407409324</v>
       </c>
       <c r="AH4">
-        <v>0.3486170929389963</v>
+        <v>0.3840185405397498</v>
       </c>
       <c r="AI4">
-        <v>0.04843587123866322</v>
+        <v>-0.1055074258040933</v>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>Suncorp Stadium</t>
+          <t>CommBank Stadium</t>
         </is>
       </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>standard_home</t>
+          <t>cross_country</t>
         </is>
       </c>
       <c r="AL4">
-        <v>1.205443668153842</v>
+        <v>1.090394280081332</v>
       </c>
       <c r="AM4">
-        <v>1.157007796915179</v>
+        <v>1.195901705885425</v>
       </c>
       <c r="AN4" t="inlineStr">
         <is>
@@ -1406,16 +1406,16 @@
         </is>
       </c>
       <c r="AP4" s="3">
-        <v>46165</v>
+        <v>46313</v>
       </c>
       <c r="AQ4" t="inlineStr">
         <is>
-          <t>2026-10-21 15:31:13 AEDT</t>
+          <t>2026-10-22 21:56:26 AEDT</t>
         </is>
       </c>
       <c r="AR4" t="inlineStr">
         <is>
-          <t>4gpo8d0qh5hhucerumdq73dhw</t>
+          <t>4hgyjdzmsg3yrculpbz3igaac</t>
         </is>
       </c>
       <c r="AS4" t="inlineStr">
@@ -1434,53 +1434,53 @@
         </is>
       </c>
       <c r="AV4" s="3">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>v046no35g7ebk8lytdjmfb43</t>
+          <t>6h553bwfqkoxayuv80uikkn42</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>cuj4qahgk4idsme4dg8clk6gw</t>
+          <t>1csft77zeexrhddgjoxuht7v8</t>
         </is>
       </c>
       <c r="AY4">
-        <v>0.37207289453206</v>
+        <v>0.3701791221391208</v>
       </c>
       <c r="AZ4">
-        <v>0.255624952906623</v>
+        <v>0.2585430038640104</v>
       </c>
       <c r="BA4">
-        <v>0.372302152561317</v>
+        <v>0.3712778739968688</v>
       </c>
       <c r="BB4">
-        <v>0.3928343032114922</v>
+        <v>0.349232980612206</v>
       </c>
       <c r="BC4">
-        <v>0.2402608253790617</v>
+        <v>0.2414127920384702</v>
       </c>
       <c r="BD4">
-        <v>0.3669048714094462</v>
+        <v>0.4093542273493238</v>
       </c>
       <c r="BE4">
-        <v>0.3722705058648712</v>
+        <v>0.3317901187193179</v>
       </c>
       <c r="BF4">
-        <v>0.2791124011961325</v>
+        <v>0.2841913407409324</v>
       </c>
       <c r="BG4">
-        <v>0.3486170929389963</v>
+        <v>0.3840185405397498</v>
       </c>
       <c r="BH4" t="b">
         <v>0</v>
       </c>
       <c r="BI4">
-        <v>0.8458305440641539</v>
+        <v>0.8297103291933792</v>
       </c>
       <c r="BJ4">
-        <v>0.9560816341569174</v>
+        <v>0.952947381716427</v>
       </c>
       <c r="BK4">
         <v>1</v>
@@ -1489,13 +1489,13 @@
         <v>1</v>
       </c>
       <c r="BM4">
-        <v>0.4736924880542347</v>
+        <v>0.5212588960967434</v>
       </c>
       <c r="BN4">
-        <v>0.4410532645932226</v>
+        <v>0.3847484432182153</v>
       </c>
       <c r="BO4">
-        <v>0.0236850596223207</v>
+        <v>0.03838900341980295</v>
       </c>
       <c r="BP4" t="b">
         <v>0</v>
@@ -1526,7 +1526,7 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <v>46319.16666666667</v>
+        <v>46319.36111111111</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1535,12 +1535,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Newcastle Jets</t>
+          <t>Melbourne Victory</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Macarthur</t>
+          <t>Melbourne City</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1569,95 +1569,95 @@
         </is>
       </c>
       <c r="K5">
-        <v>2.621779303853068</v>
+        <v>2.879826820765196</v>
       </c>
       <c r="L5">
-        <v>3.70760209890198</v>
+        <v>3.508290987165621</v>
       </c>
       <c r="M5">
-        <v>2.866450332353315</v>
+        <v>2.719476525459953</v>
       </c>
       <c r="N5">
-        <v>2.621779303853068</v>
+        <v>2.879826820765196</v>
       </c>
       <c r="O5">
-        <v>3.70760209890198</v>
+        <v>3.508290987165621</v>
       </c>
       <c r="P5">
-        <v>2.866450332353315</v>
+        <v>2.719476525459953</v>
       </c>
       <c r="Q5">
-        <v>2.683704398347222</v>
+        <v>2.696296792944173</v>
       </c>
       <c r="R5">
-        <v>3.913186147683691</v>
+        <v>3.868010859849842</v>
       </c>
       <c r="S5">
-        <v>2.68936865379867</v>
+        <v>2.698398884530992</v>
       </c>
       <c r="T5">
-        <v>2.489850097849307</v>
+        <v>2.734504521376285</v>
       </c>
       <c r="U5">
-        <v>4.293163027354093</v>
+        <v>4.060152612954442</v>
       </c>
       <c r="V5">
-        <v>2.736420572993158</v>
+        <v>2.577273914363658</v>
       </c>
       <c r="W5">
-        <v>1.760868284128208</v>
+        <v>1.545444382459734</v>
       </c>
       <c r="X5">
-        <v>1.109745545304241</v>
+        <v>1.056058773054183</v>
       </c>
       <c r="Y5">
-        <v>2.870613829432449</v>
+        <v>2.601503155513918</v>
       </c>
       <c r="Z5">
-        <v>1.374963693254859</v>
+        <v>1.347158978435769</v>
       </c>
       <c r="AA5">
-        <v>1.373247537879</v>
+        <v>1.346532733822756</v>
       </c>
       <c r="AB5">
-        <v>2.748211231133859</v>
+        <v>2.693691712258525</v>
       </c>
       <c r="AC5">
-        <v>1.656247675309587</v>
+        <v>1.439057121676726</v>
       </c>
       <c r="AD5">
-        <v>1.571192990142774</v>
+        <v>1.489241253200224</v>
       </c>
       <c r="AE5">
-        <v>3.227440665452361</v>
+        <v>2.92829837487695</v>
       </c>
       <c r="AF5">
-        <v>0.3814203577434461</v>
+        <v>0.3472431025329124</v>
       </c>
       <c r="AG5">
-        <v>0.2697161058076198</v>
+        <v>0.2850390699227343</v>
       </c>
       <c r="AH5">
-        <v>0.3488635364489341</v>
+        <v>0.3677178275443532</v>
       </c>
       <c r="AI5">
-        <v>0.06834570697379228</v>
+        <v>-0.0413005804562705</v>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>McDonald Jones Stadium</t>
+          <t>AAMI Park</t>
         </is>
       </c>
       <c r="AK5" t="inlineStr">
         <is>
-          <t>standard_home</t>
+          <t>same_city</t>
         </is>
       </c>
       <c r="AL5">
-        <v>1.285257717578417</v>
+        <v>1.119710176113525</v>
       </c>
       <c r="AM5">
-        <v>1.216912010604624</v>
+        <v>1.161010756569796</v>
       </c>
       <c r="AN5" t="inlineStr">
         <is>
@@ -1670,16 +1670,16 @@
         </is>
       </c>
       <c r="AP5" s="3">
-        <v>46165</v>
+        <v>46313</v>
       </c>
       <c r="AQ5" t="inlineStr">
         <is>
-          <t>2026-10-21 15:31:13 AEDT</t>
+          <t>2026-10-22 21:56:26 AEDT</t>
         </is>
       </c>
       <c r="AR5" t="inlineStr">
         <is>
-          <t>4h3a60ofbfqccw27euzi80qhg</t>
+          <t>4hujgxl6g64zsyrlo2clswydw</t>
         </is>
       </c>
       <c r="AS5" t="inlineStr">
@@ -1702,49 +1702,49 @@
       </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>chu9blh367xs3yumct5tqto2q</t>
+          <t>9xmhnv6im8h7c9e17oqvcx8gl</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>7jv344gvcvgqg7oeuc9u554dm</t>
+          <t>c33jm806py6adse5wv9wx6ch1</t>
         </is>
       </c>
       <c r="AY5">
-        <v>0.3726192797596698</v>
+        <v>0.3708790525645613</v>
       </c>
       <c r="AZ5">
-        <v>0.2555462383490047</v>
+        <v>0.258530814993322</v>
       </c>
       <c r="BA5">
-        <v>0.3718344818913255</v>
+        <v>0.3705901324421166</v>
       </c>
       <c r="BB5">
-        <v>0.4016306045347003</v>
+        <v>0.3656969634472196</v>
       </c>
       <c r="BC5">
-        <v>0.2329284943591595</v>
+        <v>0.2462961605948926</v>
       </c>
       <c r="BD5">
-        <v>0.3654409011061402</v>
+        <v>0.3880068759578878</v>
       </c>
       <c r="BE5">
-        <v>0.3814203577434461</v>
+        <v>0.3472431025329124</v>
       </c>
       <c r="BF5">
-        <v>0.2697161058076198</v>
+        <v>0.2850390699227343</v>
       </c>
       <c r="BG5">
-        <v>0.3488635364489341</v>
+        <v>0.3677178275443532</v>
       </c>
       <c r="BH5" t="b">
         <v>0</v>
       </c>
       <c r="BI5">
-        <v>0.9060021598260801</v>
+        <v>0.8878408610668614</v>
       </c>
       <c r="BJ5">
-        <v>0.8050226767240584</v>
+        <v>0.7865844869915635</v>
       </c>
       <c r="BK5">
         <v>1</v>
@@ -1753,13 +1753,13 @@
         <v>1</v>
       </c>
       <c r="BM5">
-        <v>0.3842705197258917</v>
+        <v>0.4390459306002075</v>
       </c>
       <c r="BN5">
-        <v>0.5123293552666615</v>
+        <v>0.4670131761020158</v>
       </c>
       <c r="BO5">
-        <v>0.02297094544239131</v>
+        <v>0.02650825492941228</v>
       </c>
       <c r="BP5" t="b">
         <v>0</v>
@@ -1790,7 +1790,7 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <v>46319.25</v>
+        <v>46320.08333333333</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1799,12 +1799,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Western Sydney Wanderers</t>
+          <t>Wellington Phoenix</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Auckland</t>
+          <t>Central Coast Mariners</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1833,83 +1833,83 @@
         </is>
       </c>
       <c r="K6">
-        <v>2.999815950034793</v>
+        <v>2.905522487158225</v>
       </c>
       <c r="L6">
-        <v>3.521886867742679</v>
+        <v>3.562858337068709</v>
       </c>
       <c r="M6">
-        <v>2.61296153189328</v>
+        <v>2.665569871360065</v>
       </c>
       <c r="N6">
-        <v>2.999815950034793</v>
+        <v>2.905522487158225</v>
       </c>
       <c r="O6">
-        <v>3.521886867742679</v>
+        <v>3.562858337068709</v>
       </c>
       <c r="P6">
-        <v>2.61296153189328</v>
+        <v>2.665569871360065</v>
       </c>
       <c r="Q6">
-        <v>2.690885574903791</v>
+        <v>2.697651636015963</v>
       </c>
       <c r="R6">
-        <v>3.911759153703458</v>
+        <v>3.868617314870624</v>
       </c>
       <c r="S6">
-        <v>2.682866385239869</v>
+        <v>2.696748520808967</v>
       </c>
       <c r="T6">
-        <v>2.848900237730245</v>
+        <v>2.763290003638433</v>
       </c>
       <c r="U6">
-        <v>4.147520281106975</v>
+        <v>4.131496118011777</v>
       </c>
       <c r="V6">
-        <v>2.451704877722552</v>
+        <v>2.524809591845969</v>
       </c>
       <c r="W6">
-        <v>1.53273790376686</v>
+        <v>1.573572320719963</v>
       </c>
       <c r="X6">
-        <v>1.101730615595587</v>
+        <v>1.093092232147512</v>
       </c>
       <c r="Y6">
-        <v>2.634468519362447</v>
+        <v>2.666664552867475</v>
       </c>
       <c r="Z6">
-        <v>1.37202440534268</v>
+        <v>1.347075246176293</v>
       </c>
       <c r="AA6">
-        <v>1.374452771237332</v>
+        <v>1.347344359149169</v>
       </c>
       <c r="AB6">
-        <v>2.746477176580012</v>
+        <v>2.694419605325463</v>
       </c>
       <c r="AC6">
-        <v>1.449726246875851</v>
+        <v>1.469300908249819</v>
       </c>
       <c r="AD6">
-        <v>1.579670591934713</v>
+        <v>1.547227625969831</v>
       </c>
       <c r="AE6">
-        <v>3.029396838810564</v>
+        <v>3.01652853421965</v>
       </c>
       <c r="AF6">
-        <v>0.3333537845841515</v>
+        <v>0.3441721770937178</v>
       </c>
       <c r="AG6">
-        <v>0.2839387060269034</v>
+        <v>0.2806735226028481</v>
       </c>
       <c r="AH6">
-        <v>0.3827075093889451</v>
+        <v>0.3751543003034342</v>
       </c>
       <c r="AI6">
-        <v>-0.09977185632449714</v>
+        <v>-0.06318098855537602</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>CommBank Stadium</t>
+          <t>Hnry Stadium</t>
         </is>
       </c>
       <c r="AK6" t="inlineStr">
@@ -1918,10 +1918,10 @@
         </is>
       </c>
       <c r="AL6">
-        <v>1.095341237588004</v>
+        <v>1.138054542300283</v>
       </c>
       <c r="AM6">
-        <v>1.195113093912501</v>
+        <v>1.201235530855659</v>
       </c>
       <c r="AN6" t="inlineStr">
         <is>
@@ -1934,16 +1934,16 @@
         </is>
       </c>
       <c r="AP6" s="3">
-        <v>46165</v>
+        <v>46313</v>
       </c>
       <c r="AQ6" t="inlineStr">
         <is>
-          <t>2026-10-21 15:31:13 AEDT</t>
+          <t>2026-10-22 21:56:26 AEDT</t>
         </is>
       </c>
       <c r="AR6" t="inlineStr">
         <is>
-          <t>4hgyjdzmsg3yrculpbz3igaac</t>
+          <t>4i7ddonqbzg9r75i3h8fdlel0</t>
         </is>
       </c>
       <c r="AS6" t="inlineStr">
@@ -1962,53 +1962,53 @@
         </is>
       </c>
       <c r="AV6" s="3">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>6h553bwfqkoxayuv80uikkn42</t>
+          <t>6j4xzc2g1eeafo6v1f38d4x22</t>
         </is>
       </c>
       <c r="AX6" t="inlineStr">
         <is>
-          <t>1csft77zeexrhddgjoxuht7v8</t>
+          <t>c4ygb6mnh53kpl2mpxe52l8jw</t>
         </is>
       </c>
       <c r="AY6">
-        <v>0.371624869272174</v>
+        <v>0.3706927857730562</v>
       </c>
       <c r="AZ6">
-        <v>0.2556394605872527</v>
+        <v>0.2584902869963612</v>
       </c>
       <c r="BA6">
-        <v>0.3727356701405733</v>
+        <v>0.3708169272305826</v>
       </c>
       <c r="BB6">
-        <v>0.351012642266727</v>
+        <v>0.3618874597611169</v>
       </c>
       <c r="BC6">
-        <v>0.2411079228606206</v>
+        <v>0.2420430690084336</v>
       </c>
       <c r="BD6">
-        <v>0.4078794348726524</v>
+        <v>0.3960694712304494</v>
       </c>
       <c r="BE6">
-        <v>0.3333537845841515</v>
+        <v>0.3441721770937178</v>
       </c>
       <c r="BF6">
-        <v>0.2839387060269034</v>
+        <v>0.2806735226028481</v>
       </c>
       <c r="BG6">
-        <v>0.3827075093889451</v>
+        <v>0.3751543003034342</v>
       </c>
       <c r="BH6" t="b">
         <v>0</v>
       </c>
       <c r="BI6">
-        <v>0.8297103291933792</v>
+        <v>0.8791943953205618</v>
       </c>
       <c r="BJ6">
-        <v>0.952947381716427</v>
+        <v>0.9055908690094202</v>
       </c>
       <c r="BK6">
         <v>1</v>
@@ -2017,13 +2017,13 @@
         <v>1</v>
       </c>
       <c r="BM6">
-        <v>0.5212588960967434</v>
+        <v>0.4511831543178876</v>
       </c>
       <c r="BN6">
-        <v>0.3847484432182153</v>
+        <v>0.4751833483035187</v>
       </c>
       <c r="BO6">
-        <v>0.03827108468802254</v>
+        <v>0.02652060867933842</v>
       </c>
       <c r="BP6" t="b">
         <v>0</v>
@@ -2054,7 +2054,7 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <v>46319.36111111111</v>
+        <v>46320.16666666667</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -2063,12 +2063,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Melbourne Victory</t>
+          <t>Sydney</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Melbourne City</t>
+          <t>Adelaide United</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -2097,95 +2097,95 @@
         </is>
       </c>
       <c r="K7">
-        <v>2.888283556771578</v>
+        <v>2.658645183516984</v>
       </c>
       <c r="L7">
-        <v>3.503018911369109</v>
+        <v>3.703130593413619</v>
       </c>
       <c r="M7">
-        <v>2.715136929903325</v>
+        <v>2.82624162481329</v>
       </c>
       <c r="N7">
-        <v>2.888283556771578</v>
+        <v>2.658645183516984</v>
       </c>
       <c r="O7">
-        <v>3.503018911369109</v>
+        <v>3.703130593413619</v>
       </c>
       <c r="P7">
-        <v>2.715136929903325</v>
+        <v>2.82624162481329</v>
       </c>
       <c r="Q7">
-        <v>2.685772770860757</v>
+        <v>2.697506714533307</v>
       </c>
       <c r="R7">
-        <v>3.911942893849746</v>
+        <v>3.867054367210901</v>
       </c>
       <c r="S7">
-        <v>2.687881368374533</v>
+        <v>2.697653439102544</v>
       </c>
       <c r="T7">
-        <v>2.74185743118545</v>
+        <v>2.530321982144931</v>
       </c>
       <c r="U7">
-        <v>4.055898700571999</v>
+        <v>4.270606193581793</v>
       </c>
       <c r="V7">
-        <v>2.572484547797126</v>
+        <v>2.69807525361021</v>
       </c>
       <c r="W7">
-        <v>1.537011350402386</v>
+        <v>1.743247895239056</v>
       </c>
       <c r="X7">
-        <v>1.055550071506222</v>
+        <v>1.112874306837603</v>
       </c>
       <c r="Y7">
-        <v>2.592561421908608</v>
+        <v>2.856122202076659</v>
       </c>
       <c r="Z7">
-        <v>1.373671236186814</v>
+        <v>1.346294111712427</v>
       </c>
       <c r="AA7">
-        <v>1.37303266700123</v>
+        <v>1.346250415979075</v>
       </c>
       <c r="AB7">
-        <v>2.746703903188044</v>
+        <v>2.692544527691502</v>
       </c>
       <c r="AC7">
-        <v>1.43434605054903</v>
+        <v>1.628885446655518</v>
       </c>
       <c r="AD7">
-        <v>1.488315576305374</v>
+        <v>1.571363885924334</v>
       </c>
       <c r="AE7">
-        <v>2.922661626854403</v>
+        <v>3.200249332579852</v>
       </c>
       <c r="AF7">
-        <v>0.346226393754</v>
+        <v>0.3761314244562533</v>
       </c>
       <c r="AG7">
-        <v>0.2854680563540444</v>
+        <v>0.2700417862061354</v>
       </c>
       <c r="AH7">
-        <v>0.3683055498919556</v>
+        <v>0.3538267893376112</v>
       </c>
       <c r="AI7">
-        <v>-0.04448835786108729</v>
+        <v>0.04678992453498299</v>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>AAMI Park</t>
+          <t>Allianz Stadium</t>
         </is>
       </c>
       <c r="AK7" t="inlineStr">
         <is>
-          <t>same_city</t>
+          <t>standard_home</t>
         </is>
       </c>
       <c r="AL7">
-        <v>1.11515511979243</v>
+        <v>1.272718891128954</v>
       </c>
       <c r="AM7">
-        <v>1.159643477653518</v>
+        <v>1.225928966593971</v>
       </c>
       <c r="AN7" t="inlineStr">
         <is>
@@ -2198,16 +2198,16 @@
         </is>
       </c>
       <c r="AP7" s="3">
-        <v>46165</v>
+        <v>46313</v>
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>2026-10-21 15:31:13 AEDT</t>
+          <t>2026-10-22 21:56:26 AEDT</t>
         </is>
       </c>
       <c r="AR7" t="inlineStr">
         <is>
-          <t>4hujgxl6g64zsyrlo2clswydw</t>
+          <t>4ik9ue5lyqnu1nhtb32a6uiac</t>
         </is>
       </c>
       <c r="AS7" t="inlineStr">
@@ -2226,53 +2226,53 @@
         </is>
       </c>
       <c r="AV7" s="3">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>9xmhnv6im8h7c9e17oqvcx8gl</t>
+          <t>38ui5tfi8anjuh533emny2tz1</t>
         </is>
       </c>
       <c r="AX7" t="inlineStr">
         <is>
-          <t>c33jm806py6adse5wv9wx6ch1</t>
+          <t>6lezh5aazy0xca1800e5dqxwl</t>
         </is>
       </c>
       <c r="AY7">
-        <v>0.372332317480273</v>
+        <v>0.3707127009591185</v>
       </c>
       <c r="AZ7">
-        <v>0.2556274534508604</v>
+        <v>0.258594761035451</v>
       </c>
       <c r="BA7">
-        <v>0.3720402290688667</v>
+        <v>0.3706925380054305</v>
       </c>
       <c r="BB7">
-        <v>0.3647162644658906</v>
+        <v>0.3952066207606942</v>
       </c>
       <c r="BC7">
-        <v>0.2465544812199011</v>
+        <v>0.2341587949511429</v>
       </c>
       <c r="BD7">
-        <v>0.3887292543142082</v>
+        <v>0.3706345842881629</v>
       </c>
       <c r="BE7">
-        <v>0.346226393754</v>
+        <v>0.3761314244562533</v>
       </c>
       <c r="BF7">
-        <v>0.2854680563540444</v>
+        <v>0.2700417862061354</v>
       </c>
       <c r="BG7">
-        <v>0.3683055498919556</v>
+        <v>0.3538267893376112</v>
       </c>
       <c r="BH7" t="b">
         <v>0</v>
       </c>
       <c r="BI7">
-        <v>0.8878408610668614</v>
+        <v>0.9632041759537114</v>
       </c>
       <c r="BJ7">
-        <v>0.7865844869915635</v>
+        <v>0.8900358093794883</v>
       </c>
       <c r="BK7">
         <v>1</v>
@@ -2281,13 +2281,13 @@
         <v>1</v>
       </c>
       <c r="BM7">
-        <v>0.4390459306002075</v>
+        <v>0.4273316030791136</v>
       </c>
       <c r="BN7">
-        <v>0.4670131761020158</v>
+        <v>0.4060941615544638</v>
       </c>
       <c r="BO7">
-        <v>0.02984060290318408</v>
+        <v>0.01686574866781931</v>
       </c>
       <c r="BP7" t="b">
         <v>0</v>
@@ -2314,11 +2314,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>ALW</t>
         </is>
       </c>
       <c r="B8" s="2">
-        <v>46320.08333333333</v>
+        <v>46319.13541666667</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -2327,129 +2327,129 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Wellington Phoenix</t>
+          <t>Western Sydney Wanderers</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Central Coast Mariners</t>
+          <t>Brisbane Roar</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Previous</t>
+          <t>Provisional</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Previous</t>
+          <t>Provisional</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Previous</t>
+          <t>Provisional</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>TEAM</t>
+          <t>PLAYER</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>previous-team fallback: TEAM is safer</t>
+          <t>reliable named teams plus material lineup change</t>
         </is>
       </c>
       <c r="K8">
-        <v>2.915664327482068</v>
+        <v>2.262167512990136</v>
       </c>
       <c r="L8">
-        <v>3.559000139457488</v>
+        <v>4.142142333373616</v>
       </c>
       <c r="M8">
-        <v>2.659240656297355</v>
+        <v>3.159306891205586</v>
       </c>
       <c r="N8">
-        <v>2.915664327482068</v>
+        <v>2.697576336274986</v>
       </c>
       <c r="O8">
-        <v>3.559000139457488</v>
+        <v>4.149874194655972</v>
       </c>
       <c r="P8">
-        <v>2.659240656297355</v>
+        <v>2.575157872597708</v>
       </c>
       <c r="Q8">
-        <v>2.687135522753262</v>
+        <v>2.262167512990136</v>
       </c>
       <c r="R8">
-        <v>3.912554241088876</v>
+        <v>4.142142333373616</v>
       </c>
       <c r="S8">
-        <v>2.686229610985881</v>
+        <v>3.159306891205586</v>
       </c>
       <c r="T8">
-        <v>2.772820637716335</v>
+        <v>2.682846116175192</v>
       </c>
       <c r="U8">
-        <v>4.128964837634106</v>
+        <v>4.270039740305243</v>
       </c>
       <c r="V8">
-        <v>2.517845535433136</v>
+        <v>2.54406540114588</v>
       </c>
       <c r="W8">
-        <v>1.565150046687582</v>
+        <v>1.536794862491703</v>
       </c>
       <c r="X8">
-        <v>1.093662397208637</v>
+        <v>1.345956992613622</v>
       </c>
       <c r="Y8">
-        <v>2.658812443896219</v>
+        <v>2.882751855105326</v>
       </c>
       <c r="Z8">
-        <v>1.373585856065965</v>
+        <v>1.630732788800927</v>
       </c>
       <c r="AA8">
-        <v>1.373860265215918</v>
+        <v>1.345436210739382</v>
       </c>
       <c r="AB8">
-        <v>2.747446121281883</v>
+        <v>2.97616899954031</v>
       </c>
       <c r="AC8">
-        <v>1.464729345059684</v>
+        <v>1.576330886528066</v>
       </c>
       <c r="AD8">
-        <v>1.547944312400016</v>
+        <v>1.623927738602791</v>
       </c>
       <c r="AE8">
-        <v>3.0126736574597</v>
+        <v>3.200258625130856</v>
       </c>
       <c r="AF8">
-        <v>0.3429750093569886</v>
+        <v>0.3707031332358418</v>
       </c>
       <c r="AG8">
-        <v>0.2809777917436198</v>
+        <v>0.2409711603517419</v>
       </c>
       <c r="AH8">
-        <v>0.3760471988993916</v>
+        <v>0.3883257064124162</v>
       </c>
       <c r="AI8">
-        <v>-0.06738801070559197</v>
+        <v>-0.04032792849581734</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>Hnry Stadium</t>
+          <t>CommBank Stadium</t>
         </is>
       </c>
       <c r="AK8" t="inlineStr">
         <is>
-          <t>cross_country</t>
+          <t>standard_home</t>
         </is>
       </c>
       <c r="AL8">
-        <v>1.133643589071108</v>
+        <v>1.501510934147084</v>
       </c>
       <c r="AM8">
-        <v>1.2010315997767</v>
+        <v>1.541838862642901</v>
       </c>
       <c r="AN8" t="inlineStr">
         <is>
@@ -2458,20 +2458,20 @@
       </c>
       <c r="AO8" t="inlineStr">
         <is>
-          <t>ALM_2026/2027_wdw_0.99_none_l0.3_total_0.99_global_l0.3</t>
+          <t>ALW_2026/2027_wdw_0.99_global_l0.02_total_0.99_global_l0.08</t>
         </is>
       </c>
       <c r="AP8" s="3">
-        <v>46165</v>
+        <v>46313</v>
       </c>
       <c r="AQ8" t="inlineStr">
         <is>
-          <t>2026-10-21 15:31:13 AEDT</t>
+          <t>2026-10-22 21:56:26 AEDT</t>
         </is>
       </c>
       <c r="AR8" t="inlineStr">
         <is>
-          <t>4i7ddonqbzg9r75i3h8fdlel0</t>
+          <t>allzuco2cijpkf76x4nae5slw</t>
         </is>
       </c>
       <c r="AS8" t="inlineStr">
@@ -2490,68 +2490,68 @@
         </is>
       </c>
       <c r="AV8" s="3">
-        <v>46320</v>
+        <v>46319</v>
       </c>
       <c r="AW8" t="inlineStr">
         <is>
-          <t>6j4xzc2g1eeafo6v1f38d4x22</t>
+          <t>loj22mimups3h7xbyfjtwsi9</t>
         </is>
       </c>
       <c r="AX8" t="inlineStr">
         <is>
-          <t>c4ygb6mnh53kpl2mpxe52l8jw</t>
+          <t>91aivk3lj1ho78ac73ulfa2sf</t>
         </is>
       </c>
       <c r="AY8">
-        <v>0.372143493148195</v>
+        <v>0.4420539125673318</v>
       </c>
       <c r="AZ8">
-        <v>0.2555875109661603</v>
+        <v>0.2414209651713099</v>
       </c>
       <c r="BA8">
-        <v>0.3722689958856447</v>
+        <v>0.3165251222613583</v>
       </c>
       <c r="BB8">
-        <v>0.360643593890584</v>
+        <v>0.3727384861811057</v>
       </c>
       <c r="BC8">
-        <v>0.242191454595433</v>
+        <v>0.2341898578977898</v>
       </c>
       <c r="BD8">
-        <v>0.3971649515139829</v>
+        <v>0.3930716559211045</v>
       </c>
       <c r="BE8">
-        <v>0.3429750093569886</v>
+        <v>0.4420539125673318</v>
       </c>
       <c r="BF8">
-        <v>0.2809777917436198</v>
+        <v>0.2414209651713099</v>
       </c>
       <c r="BG8">
-        <v>0.3760471988993916</v>
+        <v>0.3165251222613583</v>
       </c>
       <c r="BH8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BI8">
-        <v>0.8791943953205618</v>
+        <v>0.08589899229863</v>
       </c>
       <c r="BJ8">
-        <v>0.9055908690094202</v>
+        <v>0.3541735753180417</v>
       </c>
       <c r="BK8">
-        <v>1</v>
+        <v>0.9999999999999999</v>
       </c>
       <c r="BL8">
-        <v>1</v>
+        <v>0.9861354449290085</v>
       </c>
       <c r="BM8">
-        <v>0.4511831543178876</v>
+        <v>0.3770533488413551</v>
       </c>
       <c r="BN8">
-        <v>0.4751833483035187</v>
+        <v>0.5102936511248952</v>
       </c>
       <c r="BO8">
-        <v>0.0291684837912064</v>
+        <v>0.07180058415105789</v>
       </c>
       <c r="BP8" t="b">
         <v>0</v>
@@ -2578,11 +2578,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>ALW</t>
         </is>
       </c>
       <c r="B9" s="2">
-        <v>46320.16666666667</v>
+        <v>46319.16666666667</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -2591,117 +2591,117 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Sydney</t>
+          <t>Central Coast Mariners</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Adelaide United</t>
+          <t>Canberra United</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Previous</t>
+          <t>Provisional</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Previous</t>
+          <t>Provisional</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Previous</t>
+          <t>Provisional</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>TEAM</t>
+          <t>PLAYER</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>previous-team fallback: TEAM is safer</t>
+          <t>reliable named teams plus material lineup change</t>
         </is>
       </c>
       <c r="K9">
-        <v>2.654286881082492</v>
+        <v>2.259375407600953</v>
       </c>
       <c r="L9">
-        <v>3.714158771549403</v>
+        <v>4.142424936388229</v>
       </c>
       <c r="M9">
-        <v>2.824770966380978</v>
+        <v>3.164603948540582</v>
       </c>
       <c r="N9">
-        <v>2.654286881082492</v>
+        <v>2.069834047666639</v>
       </c>
       <c r="O9">
-        <v>3.714158771549403</v>
+        <v>3.968110316481232</v>
       </c>
       <c r="P9">
-        <v>2.824770966380978</v>
+        <v>3.775574461106662</v>
       </c>
       <c r="Q9">
-        <v>2.686980571331943</v>
+        <v>2.259375407600953</v>
       </c>
       <c r="R9">
-        <v>3.910978669352648</v>
+        <v>4.142424936388229</v>
       </c>
       <c r="S9">
-        <v>2.687127749641372</v>
+        <v>3.164603948540582</v>
       </c>
       <c r="T9">
-        <v>2.526830167531856</v>
+        <v>2.037998470539549</v>
       </c>
       <c r="U9">
-        <v>4.282001903413031</v>
+        <v>4.092161599085933</v>
       </c>
       <c r="V9">
-        <v>2.697514595267694</v>
+        <v>3.774256136562973</v>
       </c>
       <c r="W9">
-        <v>1.749884045315884</v>
+        <v>1.563886711454043</v>
       </c>
       <c r="X9">
-        <v>1.117405754132602</v>
+        <v>1.060653710203286</v>
       </c>
       <c r="Y9">
-        <v>2.867289799448486</v>
+        <v>2.624540421657328</v>
       </c>
       <c r="Z9">
-        <v>1.372789348777825</v>
+        <v>1.631627624248425</v>
       </c>
       <c r="AA9">
-        <v>1.372744793106957</v>
+        <v>1.34389733445913</v>
       </c>
       <c r="AB9">
-        <v>2.745534141884781</v>
+        <v>2.975524958707555</v>
       </c>
       <c r="AC9">
-        <v>1.637030473918996</v>
+        <v>1.645945228945597</v>
       </c>
       <c r="AD9">
-        <v>1.578285952005712</v>
+        <v>1.143923727080694</v>
       </c>
       <c r="AE9">
-        <v>3.215316425924708</v>
+        <v>2.789868956026291</v>
       </c>
       <c r="AF9">
-        <v>0.376749027065293</v>
+        <v>0.483130520114556</v>
       </c>
       <c r="AG9">
-        <v>0.2692399710157891</v>
+        <v>0.2520091227924232</v>
       </c>
       <c r="AH9">
-        <v>0.3540110019189179</v>
+        <v>0.2648603570930208</v>
       </c>
       <c r="AI9">
-        <v>0.04780361371979147</v>
+        <v>0.4748126518522204</v>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>Allianz Stadium</t>
+          <t>polytec Stadium</t>
         </is>
       </c>
       <c r="AK9" t="inlineStr">
@@ -2710,10 +2710,10 @@
         </is>
       </c>
       <c r="AL9">
-        <v>1.27953818685172</v>
+        <v>1.566389495876493</v>
       </c>
       <c r="AM9">
-        <v>1.231734573131928</v>
+        <v>1.091576844024273</v>
       </c>
       <c r="AN9" t="inlineStr">
         <is>
@@ -2722,20 +2722,20 @@
       </c>
       <c r="AO9" t="inlineStr">
         <is>
-          <t>ALM_2026/2027_wdw_0.99_none_l0.3_total_0.99_global_l0.3</t>
+          <t>ALW_2026/2027_wdw_0.99_global_l0.02_total_0.99_global_l0.08</t>
         </is>
       </c>
       <c r="AP9" s="3">
-        <v>46165</v>
+        <v>46313</v>
       </c>
       <c r="AQ9" t="inlineStr">
         <is>
-          <t>2026-10-21 15:31:13 AEDT</t>
+          <t>2026-10-22 21:56:26 AEDT</t>
         </is>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>4ik9ue5lyqnu1nhtb32a6uiac</t>
+          <t>alyqv0rcus6glea4xnj7amk9g</t>
         </is>
       </c>
       <c r="AS9" t="inlineStr">
@@ -2754,53 +2754,53 @@
         </is>
       </c>
       <c r="AV9" s="3">
-        <v>46320</v>
+        <v>46319</v>
       </c>
       <c r="AW9" t="inlineStr">
         <is>
-          <t>38ui5tfi8anjuh533emny2tz1</t>
+          <t>c535liylsox5safxy4qwerxx8</t>
         </is>
       </c>
       <c r="AX9" t="inlineStr">
         <is>
-          <t>6lezh5aazy0xca1800e5dqxwl</t>
+          <t>3xwecbfhkevrgr74iwq00yege</t>
         </is>
       </c>
       <c r="AY9">
-        <v>0.3721649537288234</v>
+        <v>0.4426001967781966</v>
       </c>
       <c r="AZ9">
-        <v>0.2556904766155428</v>
+        <v>0.241404495037609</v>
       </c>
       <c r="BA9">
-        <v>0.3721445696556338</v>
+        <v>0.3159953081841945</v>
       </c>
       <c r="BB9">
-        <v>0.3957527549137878</v>
+        <v>0.4906775026849041</v>
       </c>
       <c r="BC9">
-        <v>0.2335356271567595</v>
+        <v>0.2443696261221381</v>
       </c>
       <c r="BD9">
-        <v>0.3707116179294528</v>
+        <v>0.2649528711929578</v>
       </c>
       <c r="BE9">
-        <v>0.376749027065293</v>
+        <v>0.4426001967781966</v>
       </c>
       <c r="BF9">
-        <v>0.2692399710157891</v>
+        <v>0.241404495037609</v>
       </c>
       <c r="BG9">
-        <v>0.3540110019189179</v>
+        <v>0.3159953081841945</v>
       </c>
       <c r="BH9" t="b">
+        <v>1</v>
+      </c>
+      <c r="BI9">
+        <v>0.05520026134080542</v>
+      </c>
+      <c r="BJ9">
         <v>0</v>
-      </c>
-      <c r="BI9">
-        <v>0.9632041759537114</v>
-      </c>
-      <c r="BJ9">
-        <v>0.8900358093794883</v>
       </c>
       <c r="BK9">
         <v>1</v>
@@ -2809,13 +2809,13 @@
         <v>1</v>
       </c>
       <c r="BM9">
-        <v>0.4273316030791136</v>
+        <v>0.3601152553255077</v>
       </c>
       <c r="BN9">
-        <v>0.4060941615544638</v>
+        <v>0.564932682866032</v>
       </c>
       <c r="BO9">
-        <v>0.01813356773671587</v>
+        <v>0.05113495109117366</v>
       </c>
       <c r="BP9" t="b">
         <v>0</v>
@@ -2836,6 +2836,798 @@
         </is>
       </c>
       <c r="BT9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ALW</t>
+        </is>
+      </c>
+      <c r="B10" s="2">
+        <v>46319.25</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Adelaide United</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Perth Glory</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Provisional</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Provisional</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Provisional</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>TEAM/PLAYER disagreement below activation threshold</t>
+        </is>
+      </c>
+      <c r="K10">
+        <v>2.297608949742262</v>
+      </c>
+      <c r="L10">
+        <v>3.898088473424759</v>
+      </c>
+      <c r="M10">
+        <v>3.244341764748057</v>
+      </c>
+      <c r="N10">
+        <v>2.297608949742262</v>
+      </c>
+      <c r="O10">
+        <v>3.898088473424759</v>
+      </c>
+      <c r="P10">
+        <v>3.244341764748057</v>
+      </c>
+      <c r="Q10">
+        <v>2.260447104574848</v>
+      </c>
+      <c r="R10">
+        <v>4.142682152714241</v>
+      </c>
+      <c r="S10">
+        <v>3.162353949182558</v>
+      </c>
+      <c r="T10">
+        <v>2.290250956251441</v>
+      </c>
+      <c r="U10">
+        <v>4.004032778724549</v>
+      </c>
+      <c r="V10">
+        <v>3.18858820269538</v>
+      </c>
+      <c r="W10">
+        <v>1.506334184008173</v>
+      </c>
+      <c r="X10">
+        <v>1.139989636672762</v>
+      </c>
+      <c r="Y10">
+        <v>2.646323820680935</v>
+      </c>
+      <c r="Z10">
+        <v>1.631509680740385</v>
+      </c>
+      <c r="AA10">
+        <v>1.344742290052941</v>
+      </c>
+      <c r="AB10">
+        <v>2.976251970793326</v>
+      </c>
+      <c r="AC10">
+        <v>1.540210002868518</v>
+      </c>
+      <c r="AD10">
+        <v>1.267815362983758</v>
+      </c>
+      <c r="AE10">
+        <v>2.808025365852276</v>
+      </c>
+      <c r="AF10">
+        <v>0.4352350734498037</v>
+      </c>
+      <c r="AG10">
+        <v>0.2565359936844702</v>
+      </c>
+      <c r="AH10">
+        <v>0.3082289328657261</v>
+      </c>
+      <c r="AI10">
+        <v>0.2754622034306091</v>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>ServiceFM Stadium</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>standard_home</t>
+        </is>
+      </c>
+      <c r="AL10">
+        <v>1.476790036105129</v>
+      </c>
+      <c r="AM10">
+        <v>1.20132783267452</v>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>aleagues_team_player_joint_prod_v1.1.0</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>ALW_2026/2027_wdw_0.99_global_l0.02_total_0.99_global_l0.08</t>
+        </is>
+      </c>
+      <c r="AP10" s="3">
+        <v>46313</v>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>2026-10-22 21:56:26 AEDT</t>
+        </is>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>amawiescvp3380ch01vhkwh04</t>
+        </is>
+      </c>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t>Regular Season</t>
+        </is>
+      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>Fixture</t>
+        </is>
+      </c>
+      <c r="AV10" s="3">
+        <v>46319</v>
+      </c>
+      <c r="AW10" t="inlineStr">
+        <is>
+          <t>3phukn9kv66wop52orze7x414</t>
+        </is>
+      </c>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>5m9xyscemfdaoshwv8w2nfij8</t>
+        </is>
+      </c>
+      <c r="AY10">
+        <v>0.4423903563043486</v>
+      </c>
+      <c r="AZ10">
+        <v>0.2413895063961909</v>
+      </c>
+      <c r="BA10">
+        <v>0.3162201372994606</v>
+      </c>
+      <c r="BB10">
+        <v>0.4366333729805514</v>
+      </c>
+      <c r="BC10">
+        <v>0.249748205187906</v>
+      </c>
+      <c r="BD10">
+        <v>0.3136184218315426</v>
+      </c>
+      <c r="BE10">
+        <v>0.4352350734498037</v>
+      </c>
+      <c r="BF10">
+        <v>0.2565359936844702</v>
+      </c>
+      <c r="BG10">
+        <v>0.3082289328657261</v>
+      </c>
+      <c r="BH10" t="b">
+        <v>1</v>
+      </c>
+      <c r="BI10">
+        <v>0.03686647595026936</v>
+      </c>
+      <c r="BJ10">
+        <v>0.01179067958273784</v>
+      </c>
+      <c r="BK10">
+        <v>1</v>
+      </c>
+      <c r="BL10">
+        <v>1</v>
+      </c>
+      <c r="BM10">
+        <v>0.5613608914238398</v>
+      </c>
+      <c r="BN10">
+        <v>0.4902903378454601</v>
+      </c>
+      <c r="BO10">
+        <v>0.01514648728827936</v>
+      </c>
+      <c r="BP10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BQ10" t="inlineStr">
+        <is>
+          <t>aleagues_player_signal_interval_hazard_v2.0.0</t>
+        </is>
+      </c>
+      <c r="BR10" t="inlineStr">
+        <is>
+          <t>aleagues_joint_player_poisson_box_prior_v1.2.0</t>
+        </is>
+      </c>
+      <c r="BS10" t="inlineStr">
+        <is>
+          <t>aleagues_binary_team_player_router_shadow_v1.0.0</t>
+        </is>
+      </c>
+      <c r="BT10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ALW</t>
+        </is>
+      </c>
+      <c r="B11" s="2">
+        <v>46319.96875</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Wellington Phoenix</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Melbourne Victory</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Previous</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Provisional</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Previous/Provisional</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>previous-team fallback: TEAM is safer</t>
+        </is>
+      </c>
+      <c r="K11">
+        <v>2.836729214865555</v>
+      </c>
+      <c r="L11">
+        <v>3.700978256629411</v>
+      </c>
+      <c r="M11">
+        <v>2.650533736408665</v>
+      </c>
+      <c r="N11">
+        <v>2.836729214865555</v>
+      </c>
+      <c r="O11">
+        <v>3.700978256629411</v>
+      </c>
+      <c r="P11">
+        <v>2.650533736408665</v>
+      </c>
+      <c r="Q11">
+        <v>2.257955014009412</v>
+      </c>
+      <c r="R11">
+        <v>4.143337930840571</v>
+      </c>
+      <c r="S11">
+        <v>3.166861161192053</v>
+      </c>
+      <c r="T11">
+        <v>2.791223653128946</v>
+      </c>
+      <c r="U11">
+        <v>3.800278228267589</v>
+      </c>
+      <c r="V11">
+        <v>2.641341046339114</v>
+      </c>
+      <c r="W11">
+        <v>1.325755645884129</v>
+      </c>
+      <c r="X11">
+        <v>1.183486708204918</v>
+      </c>
+      <c r="Y11">
+        <v>2.509242354089047</v>
+      </c>
+      <c r="Z11">
+        <v>1.632555686877577</v>
+      </c>
+      <c r="AA11">
+        <v>1.343643924669466</v>
+      </c>
+      <c r="AB11">
+        <v>2.976199611547043</v>
+      </c>
+      <c r="AC11">
+        <v>1.284202871177841</v>
+      </c>
+      <c r="AD11">
+        <v>1.327680042942665</v>
+      </c>
+      <c r="AE11">
+        <v>2.611882914120506</v>
+      </c>
+      <c r="AF11">
+        <v>0.352518666483785</v>
+      </c>
+      <c r="AG11">
+        <v>0.2701988314059238</v>
+      </c>
+      <c r="AH11">
+        <v>0.3772825021102911</v>
+      </c>
+      <c r="AI11">
+        <v>-0.05192465401796409</v>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>Hnry Stadium</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>cross_country</t>
+        </is>
+      </c>
+      <c r="AL11">
+        <v>1.221960693441723</v>
+      </c>
+      <c r="AM11">
+        <v>1.273885347459687</v>
+      </c>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>aleagues_team_player_joint_prod_v1.1.0</t>
+        </is>
+      </c>
+      <c r="AO11" t="inlineStr">
+        <is>
+          <t>ALW_2026/2027_wdw_0.99_global_l0.02_total_0.99_global_l0.08</t>
+        </is>
+      </c>
+      <c r="AP11" s="3">
+        <v>46313</v>
+      </c>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>2026-10-22 21:56:26 AEDT</t>
+        </is>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>amxs4f3qgeq068ddj25pephck</t>
+        </is>
+      </c>
+      <c r="AS11" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="AT11" t="inlineStr">
+        <is>
+          <t>Regular Season</t>
+        </is>
+      </c>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>Fixture</t>
+        </is>
+      </c>
+      <c r="AV11" s="3">
+        <v>46320</v>
+      </c>
+      <c r="AW11" t="inlineStr">
+        <is>
+          <t>7213z0g9qz2msv8wbbi1xpzpw</t>
+        </is>
+      </c>
+      <c r="AX11" t="inlineStr">
+        <is>
+          <t>trkzv6lll4lsq6r4bafwzxp8</t>
+        </is>
+      </c>
+      <c r="AY11">
+        <v>0.442878619722506</v>
+      </c>
+      <c r="AZ11">
+        <v>0.2413513009780323</v>
+      </c>
+      <c r="BA11">
+        <v>0.3157700792994617</v>
+      </c>
+      <c r="BB11">
+        <v>0.3582658089325825</v>
+      </c>
+      <c r="BC11">
+        <v>0.2631386282619271</v>
+      </c>
+      <c r="BD11">
+        <v>0.3785955628054904</v>
+      </c>
+      <c r="BE11">
+        <v>0.352518666483785</v>
+      </c>
+      <c r="BF11">
+        <v>0.2701988314059238</v>
+      </c>
+      <c r="BG11">
+        <v>0.3772825021102911</v>
+      </c>
+      <c r="BH11" t="b">
+        <v>1</v>
+      </c>
+      <c r="BI11">
+        <v>0.957614591751602</v>
+      </c>
+      <c r="BJ11">
+        <v>0</v>
+      </c>
+      <c r="BK11">
+        <v>1</v>
+      </c>
+      <c r="BL11">
+        <v>1</v>
+      </c>
+      <c r="BM11">
+        <v>0.4568782618993489</v>
+      </c>
+      <c r="BN11">
+        <v>0.5883484054145521</v>
+      </c>
+      <c r="BO11">
+        <v>0.09035995323872098</v>
+      </c>
+      <c r="BP11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BQ11" t="inlineStr">
+        <is>
+          <t>aleagues_player_signal_interval_hazard_v2.0.0</t>
+        </is>
+      </c>
+      <c r="BR11" t="inlineStr">
+        <is>
+          <t>aleagues_joint_player_poisson_box_prior_v1.2.0</t>
+        </is>
+      </c>
+      <c r="BS11" t="inlineStr">
+        <is>
+          <t>aleagues_binary_team_player_router_shadow_v1.0.0</t>
+        </is>
+      </c>
+      <c r="BT11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ALW</t>
+        </is>
+      </c>
+      <c r="B12" s="2">
+        <v>46320.28125</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Melbourne City</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Provisional</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Previous</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Provisional/Previous</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>previous-team fallback: TEAM is safer</t>
+        </is>
+      </c>
+      <c r="K12">
+        <v>3.350471225096801</v>
+      </c>
+      <c r="L12">
+        <v>3.685580484121762</v>
+      </c>
+      <c r="M12">
+        <v>2.324463267306392</v>
+      </c>
+      <c r="N12">
+        <v>3.350471225096801</v>
+      </c>
+      <c r="O12">
+        <v>3.685580484121762</v>
+      </c>
+      <c r="P12">
+        <v>2.324463267306392</v>
+      </c>
+      <c r="Q12">
+        <v>2.263931179100951</v>
+      </c>
+      <c r="R12">
+        <v>4.140577967855312</v>
+      </c>
+      <c r="S12">
+        <v>3.156782061103599</v>
+      </c>
+      <c r="T12">
+        <v>3.300744134823141</v>
+      </c>
+      <c r="U12">
+        <v>3.782517800277875</v>
+      </c>
+      <c r="V12">
+        <v>2.311263149427268</v>
+      </c>
+      <c r="W12">
+        <v>1.216016271245613</v>
+      </c>
+      <c r="X12">
+        <v>1.258340109812224</v>
+      </c>
+      <c r="Y12">
+        <v>2.474356381057836</v>
+      </c>
+      <c r="Z12">
+        <v>1.629313332120638</v>
+      </c>
+      <c r="AA12">
+        <v>1.345443767711301</v>
+      </c>
+      <c r="AB12">
+        <v>2.974757099831939</v>
+      </c>
+      <c r="AC12">
+        <v>1.133474330293256</v>
+      </c>
+      <c r="AD12">
+        <v>1.408464040755703</v>
+      </c>
+      <c r="AE12">
+        <v>2.54193837104896</v>
+      </c>
+      <c r="AF12">
+        <v>0.2984654792763093</v>
+      </c>
+      <c r="AG12">
+        <v>0.2713276794003565</v>
+      </c>
+      <c r="AH12">
+        <v>0.4302068413233342</v>
+      </c>
+      <c r="AI12">
+        <v>-0.2739921127482854</v>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>Allianz Stadium</t>
+        </is>
+      </c>
+      <c r="AK12" t="inlineStr">
+        <is>
+          <t>standard_home</t>
+        </is>
+      </c>
+      <c r="AL12">
+        <v>1.078565494444899</v>
+      </c>
+      <c r="AM12">
+        <v>1.352557607193185</v>
+      </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>aleagues_team_player_joint_prod_v1.1.0</t>
+        </is>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>ALW_2026/2027_wdw_0.99_global_l0.02_total_0.99_global_l0.08</t>
+        </is>
+      </c>
+      <c r="AP12" s="3">
+        <v>46313</v>
+      </c>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>2026-10-22 21:56:26 AEDT</t>
+        </is>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>ammlv3t3xtze8gagdmzt5wtg4</t>
+        </is>
+      </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>Regular Season</t>
+        </is>
+      </c>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>Fixture</t>
+        </is>
+      </c>
+      <c r="AV12" s="3">
+        <v>46320</v>
+      </c>
+      <c r="AW12" t="inlineStr">
+        <is>
+          <t>ezzu9xtrjsagi3id3hjrcizf1</t>
+        </is>
+      </c>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>6l09hlipvei5y89k8eist1gh</t>
+        </is>
+      </c>
+      <c r="AY12">
+        <v>0.4417095401270626</v>
+      </c>
+      <c r="AZ12">
+        <v>0.2415121772282357</v>
+      </c>
+      <c r="BA12">
+        <v>0.3167782826447017</v>
+      </c>
+      <c r="BB12">
+        <v>0.302961986495685</v>
+      </c>
+      <c r="BC12">
+        <v>0.2643741689534249</v>
+      </c>
+      <c r="BD12">
+        <v>0.4326638445508901</v>
+      </c>
+      <c r="BE12">
+        <v>0.2984654792763093</v>
+      </c>
+      <c r="BF12">
+        <v>0.2713276794003565</v>
+      </c>
+      <c r="BG12">
+        <v>0.4302068413233342</v>
+      </c>
+      <c r="BH12" t="b">
+        <v>1</v>
+      </c>
+      <c r="BI12">
+        <v>0.06349047801555961</v>
+      </c>
+      <c r="BJ12">
+        <v>0.956941732530076</v>
+      </c>
+      <c r="BK12">
+        <v>1</v>
+      </c>
+      <c r="BL12">
+        <v>1</v>
+      </c>
+      <c r="BM12">
+        <v>0.7703956100310558</v>
+      </c>
+      <c r="BN12">
+        <v>0.3883313560910396</v>
+      </c>
+      <c r="BO12">
+        <v>0.1432440608507533</v>
+      </c>
+      <c r="BP12" t="b">
+        <v>1</v>
+      </c>
+      <c r="BQ12" t="inlineStr">
+        <is>
+          <t>aleagues_player_signal_interval_hazard_v2.0.0</t>
+        </is>
+      </c>
+      <c r="BR12" t="inlineStr">
+        <is>
+          <t>aleagues_joint_player_poisson_box_prior_v1.2.0</t>
+        </is>
+      </c>
+      <c r="BS12" t="inlineStr">
+        <is>
+          <t>aleagues_binary_team_player_router_shadow_v1.0.0</t>
+        </is>
+      </c>
+      <c r="BT12" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>